<commit_message>
InteliNeo register map from the controller's Modbus export; inverter profile with SAU signal IDs (registers pending); plant PC and controller inventory; adapter bit masks, derived sums, address offset
</commit_message>
<xml_diff>
--- a/docs/turkey/Solar_Inverter_Tag_List_Rev.1.2.xlsx
+++ b/docs/turkey/Solar_Inverter_Tag_List_Rev.1.2.xlsx
@@ -1095,7 +1095,7 @@
       </c>
       <c r="K2" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1000</t>
+          <t>Pending - register map of the source device not yet available - quality register 1000</t>
         </is>
       </c>
       <c r="L2" s="5" t="inlineStr">
@@ -1151,7 +1151,7 @@
       </c>
       <c r="K3" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1001</t>
+          <t>Pending - register map of the source device not yet available - quality register 1001</t>
         </is>
       </c>
       <c r="L3" s="5" t="inlineStr">
@@ -1207,7 +1207,7 @@
       </c>
       <c r="K4" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1002</t>
+          <t>Pending - register map of the source device not yet available - quality register 1002</t>
         </is>
       </c>
       <c r="L4" s="5" t="inlineStr">
@@ -1263,7 +1263,7 @@
       </c>
       <c r="K5" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1003</t>
+          <t>Pending - register map of the source device not yet available - quality register 1003</t>
         </is>
       </c>
       <c r="L5" s="5" t="inlineStr">
@@ -1319,7 +1319,7 @@
       </c>
       <c r="K6" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1004</t>
+          <t>Pending - register map of the source device not yet available - quality register 1004</t>
         </is>
       </c>
       <c r="L6" s="5" t="inlineStr">
@@ -1375,7 +1375,7 @@
       </c>
       <c r="K7" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1005</t>
+          <t>Pending - register map of the source device not yet available - quality register 1005</t>
         </is>
       </c>
       <c r="L7" s="5" t="inlineStr">
@@ -1431,7 +1431,7 @@
       </c>
       <c r="K8" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1006</t>
+          <t>Pending - register map of the source device not yet available - quality register 1006</t>
         </is>
       </c>
       <c r="L8" s="5" t="inlineStr">
@@ -1487,7 +1487,7 @@
       </c>
       <c r="K9" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1007</t>
+          <t>Pending - register map of the source device not yet available - quality register 1007</t>
         </is>
       </c>
       <c r="L9" s="5" t="inlineStr">
@@ -1543,7 +1543,7 @@
       </c>
       <c r="K10" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1008</t>
+          <t>Pending - register map of the source device not yet available - quality register 1008</t>
         </is>
       </c>
       <c r="L10" s="5" t="inlineStr">
@@ -1599,7 +1599,7 @@
       </c>
       <c r="K11" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1009</t>
+          <t>Pending - register map of the source device not yet available - quality register 1009</t>
         </is>
       </c>
       <c r="L11" s="5" t="inlineStr">
@@ -1651,7 +1651,7 @@
       </c>
       <c r="K12" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1010</t>
+          <t>Pending - register map of the source device not yet available - quality register 1010</t>
         </is>
       </c>
       <c r="L12" s="5" t="inlineStr">
@@ -1707,7 +1707,7 @@
       </c>
       <c r="K13" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1011</t>
+          <t>Pending - register map of the source device not yet available - quality register 1011</t>
         </is>
       </c>
       <c r="L13" s="5" t="inlineStr">
@@ -1763,7 +1763,7 @@
       </c>
       <c r="K14" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1012</t>
+          <t>Pending - register map of the source device not yet available - quality register 1012</t>
         </is>
       </c>
       <c r="L14" s="5" t="inlineStr">
@@ -1819,7 +1819,7 @@
       </c>
       <c r="K15" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1013</t>
+          <t>Pending - register map of the source device not yet available - quality register 1013</t>
         </is>
       </c>
       <c r="L15" s="5" t="inlineStr">
@@ -1875,7 +1875,7 @@
       </c>
       <c r="K16" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1014</t>
+          <t>Pending - register map of the source device not yet available - quality register 1014</t>
         </is>
       </c>
       <c r="L16" s="5" t="inlineStr">
@@ -1931,7 +1931,7 @@
       </c>
       <c r="K17" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1015</t>
+          <t>Pending - register map of the source device not yet available - quality register 1015</t>
         </is>
       </c>
       <c r="L17" s="5" t="inlineStr">
@@ -1987,7 +1987,7 @@
       </c>
       <c r="K18" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1016</t>
+          <t>Pending - register map of the source device not yet available - quality register 1016</t>
         </is>
       </c>
       <c r="L18" s="5" t="inlineStr">
@@ -2043,7 +2043,7 @@
       </c>
       <c r="K19" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1017</t>
+          <t>Pending - register map of the source device not yet available - quality register 1017</t>
         </is>
       </c>
       <c r="L19" s="5" t="inlineStr">
@@ -2099,7 +2099,7 @@
       </c>
       <c r="K20" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1018</t>
+          <t>Pending - register map of the source device not yet available - quality register 1018</t>
         </is>
       </c>
       <c r="L20" s="5" t="inlineStr">
@@ -2155,7 +2155,7 @@
       </c>
       <c r="K21" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1019</t>
+          <t>Pending - register map of the source device not yet available - quality register 1019</t>
         </is>
       </c>
       <c r="L21" s="5" t="inlineStr">
@@ -2211,7 +2211,7 @@
       </c>
       <c r="K22" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1020</t>
+          <t>Pending - register map of the source device not yet available - quality register 1020</t>
         </is>
       </c>
       <c r="L22" s="5" t="inlineStr">
@@ -2267,7 +2267,7 @@
       </c>
       <c r="K23" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1021</t>
+          <t>Pending - register map of the source device not yet available - quality register 1021</t>
         </is>
       </c>
       <c r="L23" s="5" t="inlineStr">
@@ -2323,7 +2323,7 @@
       </c>
       <c r="K24" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1022</t>
+          <t>Pending - register map of the source device not yet available - quality register 1022</t>
         </is>
       </c>
       <c r="L24" s="5" t="inlineStr">
@@ -2379,7 +2379,7 @@
       </c>
       <c r="K25" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1023</t>
+          <t>Pending - register map of the source device not yet available - quality register 1023</t>
         </is>
       </c>
       <c r="L25" s="5" t="inlineStr">
@@ -2435,7 +2435,7 @@
       </c>
       <c r="K26" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1024</t>
+          <t>Pending - register map of the source device not yet available - quality register 1024</t>
         </is>
       </c>
       <c r="L26" s="5" t="inlineStr">
@@ -2491,7 +2491,7 @@
       </c>
       <c r="K27" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1025</t>
+          <t>Pending - register map of the source device not yet available - quality register 1025</t>
         </is>
       </c>
       <c r="L27" s="5" t="inlineStr">
@@ -2547,7 +2547,7 @@
       </c>
       <c r="K28" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1026</t>
+          <t>Pending - register map of the source device not yet available - quality register 1026</t>
         </is>
       </c>
       <c r="L28" s="5" t="inlineStr">
@@ -2603,7 +2603,7 @@
       </c>
       <c r="K29" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1027</t>
+          <t>Pending - register map of the source device not yet available - quality register 1027</t>
         </is>
       </c>
       <c r="L29" s="5" t="inlineStr">
@@ -2659,7 +2659,7 @@
       </c>
       <c r="K30" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1028</t>
+          <t>Pending - register map of the source device not yet available - quality register 1028</t>
         </is>
       </c>
       <c r="L30" s="5" t="inlineStr">
@@ -2715,7 +2715,7 @@
       </c>
       <c r="K31" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1029</t>
+          <t>Pending - register map of the source device not yet available - quality register 1029</t>
         </is>
       </c>
       <c r="L31" s="5" t="inlineStr">
@@ -2771,7 +2771,7 @@
       </c>
       <c r="K32" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1030</t>
+          <t>Pending - register map of the source device not yet available - quality register 1030</t>
         </is>
       </c>
       <c r="L32" s="5" t="inlineStr">
@@ -2827,7 +2827,7 @@
       </c>
       <c r="K33" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1031</t>
+          <t>Pending - register map of the source device not yet available - quality register 1031</t>
         </is>
       </c>
       <c r="L33" s="5" t="inlineStr">
@@ -2883,7 +2883,7 @@
       </c>
       <c r="K34" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1032</t>
+          <t>Pending - register map of the source device not yet available - quality register 1032</t>
         </is>
       </c>
       <c r="L34" s="5" t="inlineStr">
@@ -2939,7 +2939,7 @@
       </c>
       <c r="K35" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1033</t>
+          <t>Pending - register map of the source device not yet available - quality register 1033</t>
         </is>
       </c>
       <c r="L35" s="5" t="inlineStr">
@@ -2995,7 +2995,7 @@
       </c>
       <c r="K36" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1034</t>
+          <t>Pending - register map of the source device not yet available - quality register 1034</t>
         </is>
       </c>
       <c r="L36" s="5" t="inlineStr">
@@ -3051,7 +3051,7 @@
       </c>
       <c r="K37" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1035</t>
+          <t>Pending - register map of the source device not yet available - quality register 1035</t>
         </is>
       </c>
       <c r="L37" s="5" t="inlineStr">
@@ -3107,7 +3107,7 @@
       </c>
       <c r="K38" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1036</t>
+          <t>Pending - register map of the source device not yet available - quality register 1036</t>
         </is>
       </c>
       <c r="L38" s="5" t="inlineStr">
@@ -3163,7 +3163,7 @@
       </c>
       <c r="K39" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1037</t>
+          <t>Pending - register map of the source device not yet available - quality register 1037</t>
         </is>
       </c>
       <c r="L39" s="5" t="inlineStr">
@@ -3219,7 +3219,7 @@
       </c>
       <c r="K40" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1038</t>
+          <t>Pending - register map of the source device not yet available - quality register 1038</t>
         </is>
       </c>
       <c r="L40" s="5" t="inlineStr">
@@ -3271,7 +3271,7 @@
       </c>
       <c r="K41" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1039</t>
+          <t>Pending - register map of the source device not yet available - quality register 1039</t>
         </is>
       </c>
       <c r="L41" s="5" t="inlineStr">
@@ -3327,7 +3327,7 @@
       </c>
       <c r="K42" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1040</t>
+          <t>Pending - register map of the source device not yet available - quality register 1040</t>
         </is>
       </c>
       <c r="L42" s="5" t="inlineStr">
@@ -3383,7 +3383,7 @@
       </c>
       <c r="K43" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1041</t>
+          <t>Pending - register map of the source device not yet available - quality register 1041</t>
         </is>
       </c>
       <c r="L43" s="5" t="inlineStr">
@@ -3439,7 +3439,7 @@
       </c>
       <c r="K44" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1042</t>
+          <t>Pending - register map of the source device not yet available - quality register 1042</t>
         </is>
       </c>
       <c r="L44" s="5" t="inlineStr">
@@ -3495,7 +3495,7 @@
       </c>
       <c r="K45" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1043</t>
+          <t>Pending - register map of the source device not yet available - quality register 1043</t>
         </is>
       </c>
       <c r="L45" s="5" t="inlineStr">
@@ -3551,7 +3551,7 @@
       </c>
       <c r="K46" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1044</t>
+          <t>Pending - register map of the source device not yet available - quality register 1044</t>
         </is>
       </c>
       <c r="L46" s="5" t="inlineStr">
@@ -3607,7 +3607,7 @@
       </c>
       <c r="K47" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1045</t>
+          <t>Pending - register map of the source device not yet available - quality register 1045</t>
         </is>
       </c>
       <c r="L47" s="5" t="inlineStr">
@@ -3663,7 +3663,7 @@
       </c>
       <c r="K48" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1046</t>
+          <t>Pending - register map of the source device not yet available - quality register 1046</t>
         </is>
       </c>
       <c r="L48" s="5" t="inlineStr">
@@ -3719,7 +3719,7 @@
       </c>
       <c r="K49" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1047</t>
+          <t>Pending - register map of the source device not yet available - quality register 1047</t>
         </is>
       </c>
       <c r="L49" s="5" t="inlineStr">
@@ -3775,7 +3775,7 @@
       </c>
       <c r="K50" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1048</t>
+          <t>Pending - register map of the source device not yet available - quality register 1048</t>
         </is>
       </c>
       <c r="L50" s="5" t="inlineStr">
@@ -3831,7 +3831,7 @@
       </c>
       <c r="K51" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1049</t>
+          <t>Pending - register map of the source device not yet available - quality register 1049</t>
         </is>
       </c>
       <c r="L51" s="5" t="inlineStr">
@@ -3887,7 +3887,7 @@
       </c>
       <c r="K52" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1050</t>
+          <t>Pending - register map of the source device not yet available - quality register 1050</t>
         </is>
       </c>
       <c r="L52" s="5" t="inlineStr">
@@ -3943,7 +3943,7 @@
       </c>
       <c r="K53" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1051</t>
+          <t>Pending - register map of the source device not yet available - quality register 1051</t>
         </is>
       </c>
       <c r="L53" s="5" t="inlineStr">
@@ -3999,7 +3999,7 @@
       </c>
       <c r="K54" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1052</t>
+          <t>Pending - register map of the source device not yet available - quality register 1052</t>
         </is>
       </c>
       <c r="L54" s="5" t="inlineStr">
@@ -4055,7 +4055,7 @@
       </c>
       <c r="K55" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1053</t>
+          <t>Pending - register map of the source device not yet available - quality register 1053</t>
         </is>
       </c>
       <c r="L55" s="5" t="inlineStr">
@@ -4111,7 +4111,7 @@
       </c>
       <c r="K56" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1054</t>
+          <t>Pending - register map of the source device not yet available - quality register 1054</t>
         </is>
       </c>
       <c r="L56" s="5" t="inlineStr">
@@ -4167,7 +4167,7 @@
       </c>
       <c r="K57" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1055</t>
+          <t>Pending - register map of the source device not yet available - quality register 1055</t>
         </is>
       </c>
       <c r="L57" s="5" t="inlineStr">
@@ -4223,7 +4223,7 @@
       </c>
       <c r="K58" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1056</t>
+          <t>Pending - register map of the source device not yet available - quality register 1056</t>
         </is>
       </c>
       <c r="L58" s="5" t="inlineStr">
@@ -4279,7 +4279,7 @@
       </c>
       <c r="K59" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1057</t>
+          <t>Pending - register map of the source device not yet available - quality register 1057</t>
         </is>
       </c>
       <c r="L59" s="5" t="inlineStr">
@@ -4335,7 +4335,7 @@
       </c>
       <c r="K60" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1058</t>
+          <t>Pending - register map of the source device not yet available - quality register 1058</t>
         </is>
       </c>
       <c r="L60" s="5" t="inlineStr">
@@ -4391,7 +4391,7 @@
       </c>
       <c r="K61" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1059</t>
+          <t>Pending - register map of the source device not yet available - quality register 1059</t>
         </is>
       </c>
       <c r="L61" s="5" t="inlineStr">
@@ -4447,7 +4447,7 @@
       </c>
       <c r="K62" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1060</t>
+          <t>Pending - register map of the source device not yet available - quality register 1060</t>
         </is>
       </c>
       <c r="L62" s="5" t="inlineStr">
@@ -4503,7 +4503,7 @@
       </c>
       <c r="K63" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1061</t>
+          <t>Pending - register map of the source device not yet available - quality register 1061</t>
         </is>
       </c>
       <c r="L63" s="5" t="inlineStr">
@@ -4559,7 +4559,7 @@
       </c>
       <c r="K64" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1062</t>
+          <t>Pending - register map of the source device not yet available - quality register 1062</t>
         </is>
       </c>
       <c r="L64" s="5" t="inlineStr">
@@ -4615,7 +4615,7 @@
       </c>
       <c r="K65" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1063</t>
+          <t>Pending - register map of the source device not yet available - quality register 1063</t>
         </is>
       </c>
       <c r="L65" s="5" t="inlineStr">
@@ -4671,7 +4671,7 @@
       </c>
       <c r="K66" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1064</t>
+          <t>Pending - register map of the source device not yet available - quality register 1064</t>
         </is>
       </c>
       <c r="L66" s="5" t="inlineStr">
@@ -4727,7 +4727,7 @@
       </c>
       <c r="K67" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1065</t>
+          <t>Pending - register map of the source device not yet available - quality register 1065</t>
         </is>
       </c>
       <c r="L67" s="5" t="inlineStr">
@@ -4783,7 +4783,7 @@
       </c>
       <c r="K68" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1066</t>
+          <t>Pending - register map of the source device not yet available - quality register 1066</t>
         </is>
       </c>
       <c r="L68" s="5" t="inlineStr">
@@ -4839,7 +4839,7 @@
       </c>
       <c r="K69" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1067</t>
+          <t>Pending - register map of the source device not yet available - quality register 1067</t>
         </is>
       </c>
       <c r="L69" s="5" t="inlineStr">
@@ -4891,7 +4891,7 @@
       </c>
       <c r="K70" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1068</t>
+          <t>Pending - register map of the source device not yet available - quality register 1068</t>
         </is>
       </c>
       <c r="L70" s="5" t="inlineStr">
@@ -4947,7 +4947,7 @@
       </c>
       <c r="K71" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1069</t>
+          <t>Pending - register map of the source device not yet available - quality register 1069</t>
         </is>
       </c>
       <c r="L71" s="5" t="inlineStr">
@@ -5003,7 +5003,7 @@
       </c>
       <c r="K72" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1070</t>
+          <t>Pending - register map of the source device not yet available - quality register 1070</t>
         </is>
       </c>
       <c r="L72" s="5" t="inlineStr">
@@ -5059,7 +5059,7 @@
       </c>
       <c r="K73" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1071</t>
+          <t>Pending - register map of the source device not yet available - quality register 1071</t>
         </is>
       </c>
       <c r="L73" s="5" t="inlineStr">
@@ -5115,7 +5115,7 @@
       </c>
       <c r="K74" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1072</t>
+          <t>Pending - register map of the source device not yet available - quality register 1072</t>
         </is>
       </c>
       <c r="L74" s="5" t="inlineStr">
@@ -5171,7 +5171,7 @@
       </c>
       <c r="K75" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1073</t>
+          <t>Pending - register map of the source device not yet available - quality register 1073</t>
         </is>
       </c>
       <c r="L75" s="5" t="inlineStr">
@@ -5227,7 +5227,7 @@
       </c>
       <c r="K76" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1074</t>
+          <t>Pending - register map of the source device not yet available - quality register 1074</t>
         </is>
       </c>
       <c r="L76" s="5" t="inlineStr">
@@ -5283,7 +5283,7 @@
       </c>
       <c r="K77" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1075</t>
+          <t>Pending - register map of the source device not yet available - quality register 1075</t>
         </is>
       </c>
       <c r="L77" s="5" t="inlineStr">
@@ -5339,7 +5339,7 @@
       </c>
       <c r="K78" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1076</t>
+          <t>Pending - register map of the source device not yet available - quality register 1076</t>
         </is>
       </c>
       <c r="L78" s="5" t="inlineStr">
@@ -5395,7 +5395,7 @@
       </c>
       <c r="K79" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1077</t>
+          <t>Pending - register map of the source device not yet available - quality register 1077</t>
         </is>
       </c>
       <c r="L79" s="5" t="inlineStr">
@@ -5451,7 +5451,7 @@
       </c>
       <c r="K80" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1078</t>
+          <t>Pending - register map of the source device not yet available - quality register 1078</t>
         </is>
       </c>
       <c r="L80" s="5" t="inlineStr">
@@ -5507,7 +5507,7 @@
       </c>
       <c r="K81" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1079</t>
+          <t>Pending - register map of the source device not yet available - quality register 1079</t>
         </is>
       </c>
       <c r="L81" s="5" t="inlineStr">
@@ -5563,7 +5563,7 @@
       </c>
       <c r="K82" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1080</t>
+          <t>Pending - register map of the source device not yet available - quality register 1080</t>
         </is>
       </c>
       <c r="L82" s="5" t="inlineStr">
@@ -5619,7 +5619,7 @@
       </c>
       <c r="K83" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1081</t>
+          <t>Pending - register map of the source device not yet available - quality register 1081</t>
         </is>
       </c>
       <c r="L83" s="5" t="inlineStr">
@@ -5675,7 +5675,7 @@
       </c>
       <c r="K84" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1082</t>
+          <t>Pending - register map of the source device not yet available - quality register 1082</t>
         </is>
       </c>
       <c r="L84" s="5" t="inlineStr">
@@ -5731,7 +5731,7 @@
       </c>
       <c r="K85" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1083</t>
+          <t>Pending - register map of the source device not yet available - quality register 1083</t>
         </is>
       </c>
       <c r="L85" s="5" t="inlineStr">
@@ -5787,7 +5787,7 @@
       </c>
       <c r="K86" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1084</t>
+          <t>Pending - register map of the source device not yet available - quality register 1084</t>
         </is>
       </c>
       <c r="L86" s="5" t="inlineStr">
@@ -5843,7 +5843,7 @@
       </c>
       <c r="K87" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1085</t>
+          <t>Pending - register map of the source device not yet available - quality register 1085</t>
         </is>
       </c>
       <c r="L87" s="5" t="inlineStr">
@@ -5899,7 +5899,7 @@
       </c>
       <c r="K88" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1086</t>
+          <t>Pending - register map of the source device not yet available - quality register 1086</t>
         </is>
       </c>
       <c r="L88" s="5" t="inlineStr">
@@ -5955,7 +5955,7 @@
       </c>
       <c r="K89" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1087</t>
+          <t>Pending - register map of the source device not yet available - quality register 1087</t>
         </is>
       </c>
       <c r="L89" s="5" t="inlineStr">
@@ -6011,7 +6011,7 @@
       </c>
       <c r="K90" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1088</t>
+          <t>Pending - register map of the source device not yet available - quality register 1088</t>
         </is>
       </c>
       <c r="L90" s="5" t="inlineStr">
@@ -6067,7 +6067,7 @@
       </c>
       <c r="K91" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1089</t>
+          <t>Pending - register map of the source device not yet available - quality register 1089</t>
         </is>
       </c>
       <c r="L91" s="5" t="inlineStr">
@@ -6123,7 +6123,7 @@
       </c>
       <c r="K92" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1090</t>
+          <t>Pending - register map of the source device not yet available - quality register 1090</t>
         </is>
       </c>
       <c r="L92" s="5" t="inlineStr">
@@ -6179,7 +6179,7 @@
       </c>
       <c r="K93" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1091</t>
+          <t>Pending - register map of the source device not yet available - quality register 1091</t>
         </is>
       </c>
       <c r="L93" s="5" t="inlineStr">
@@ -6235,7 +6235,7 @@
       </c>
       <c r="K94" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1092</t>
+          <t>Pending - register map of the source device not yet available - quality register 1092</t>
         </is>
       </c>
       <c r="L94" s="5" t="inlineStr">
@@ -6291,7 +6291,7 @@
       </c>
       <c r="K95" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1093</t>
+          <t>Pending - register map of the source device not yet available - quality register 1093</t>
         </is>
       </c>
       <c r="L95" s="5" t="inlineStr">
@@ -6347,7 +6347,7 @@
       </c>
       <c r="K96" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1094</t>
+          <t>Pending - register map of the source device not yet available - quality register 1094</t>
         </is>
       </c>
       <c r="L96" s="5" t="inlineStr">
@@ -6403,7 +6403,7 @@
       </c>
       <c r="K97" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1095</t>
+          <t>Pending - register map of the source device not yet available - quality register 1095</t>
         </is>
       </c>
       <c r="L97" s="5" t="inlineStr">
@@ -6459,7 +6459,7 @@
       </c>
       <c r="K98" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1096</t>
+          <t>Pending - register map of the source device not yet available - quality register 1096</t>
         </is>
       </c>
       <c r="L98" s="5" t="inlineStr">
@@ -6511,7 +6511,7 @@
       </c>
       <c r="K99" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1097</t>
+          <t>Pending - register map of the source device not yet available - quality register 1097</t>
         </is>
       </c>
       <c r="L99" s="5" t="inlineStr">
@@ -6567,7 +6567,7 @@
       </c>
       <c r="K100" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1098</t>
+          <t>Pending - register map of the source device not yet available - quality register 1098</t>
         </is>
       </c>
       <c r="L100" s="5" t="inlineStr">
@@ -6623,7 +6623,7 @@
       </c>
       <c r="K101" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1099</t>
+          <t>Pending - register map of the source device not yet available - quality register 1099</t>
         </is>
       </c>
       <c r="L101" s="5" t="inlineStr">
@@ -6679,7 +6679,7 @@
       </c>
       <c r="K102" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1100</t>
+          <t>Pending - register map of the source device not yet available - quality register 1100</t>
         </is>
       </c>
       <c r="L102" s="5" t="inlineStr">
@@ -6735,7 +6735,7 @@
       </c>
       <c r="K103" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1101</t>
+          <t>Pending - register map of the source device not yet available - quality register 1101</t>
         </is>
       </c>
       <c r="L103" s="5" t="inlineStr">
@@ -6791,7 +6791,7 @@
       </c>
       <c r="K104" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1102</t>
+          <t>Pending - register map of the source device not yet available - quality register 1102</t>
         </is>
       </c>
       <c r="L104" s="5" t="inlineStr">
@@ -6847,7 +6847,7 @@
       </c>
       <c r="K105" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1103</t>
+          <t>Pending - register map of the source device not yet available - quality register 1103</t>
         </is>
       </c>
       <c r="L105" s="5" t="inlineStr">
@@ -6903,7 +6903,7 @@
       </c>
       <c r="K106" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1104</t>
+          <t>Pending - register map of the source device not yet available - quality register 1104</t>
         </is>
       </c>
       <c r="L106" s="5" t="inlineStr">
@@ -6959,7 +6959,7 @@
       </c>
       <c r="K107" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1105</t>
+          <t>Pending - register map of the source device not yet available - quality register 1105</t>
         </is>
       </c>
       <c r="L107" s="5" t="inlineStr">
@@ -7015,7 +7015,7 @@
       </c>
       <c r="K108" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1106</t>
+          <t>Pending - register map of the source device not yet available - quality register 1106</t>
         </is>
       </c>
       <c r="L108" s="5" t="inlineStr">
@@ -7071,7 +7071,7 @@
       </c>
       <c r="K109" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1107</t>
+          <t>Pending - register map of the source device not yet available - quality register 1107</t>
         </is>
       </c>
       <c r="L109" s="5" t="inlineStr">
@@ -7127,7 +7127,7 @@
       </c>
       <c r="K110" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1108</t>
+          <t>Pending - register map of the source device not yet available - quality register 1108</t>
         </is>
       </c>
       <c r="L110" s="5" t="inlineStr">
@@ -7183,7 +7183,7 @@
       </c>
       <c r="K111" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1109</t>
+          <t>Pending - register map of the source device not yet available - quality register 1109</t>
         </is>
       </c>
       <c r="L111" s="5" t="inlineStr">
@@ -7239,7 +7239,7 @@
       </c>
       <c r="K112" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1110</t>
+          <t>Pending - register map of the source device not yet available - quality register 1110</t>
         </is>
       </c>
       <c r="L112" s="5" t="inlineStr">
@@ -7295,7 +7295,7 @@
       </c>
       <c r="K113" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1111</t>
+          <t>Pending - register map of the source device not yet available - quality register 1111</t>
         </is>
       </c>
       <c r="L113" s="5" t="inlineStr">
@@ -7351,7 +7351,7 @@
       </c>
       <c r="K114" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1112</t>
+          <t>Pending - register map of the source device not yet available - quality register 1112</t>
         </is>
       </c>
       <c r="L114" s="5" t="inlineStr">
@@ -7407,7 +7407,7 @@
       </c>
       <c r="K115" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1113</t>
+          <t>Pending - register map of the source device not yet available - quality register 1113</t>
         </is>
       </c>
       <c r="L115" s="5" t="inlineStr">
@@ -7463,7 +7463,7 @@
       </c>
       <c r="K116" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1114</t>
+          <t>Pending - register map of the source device not yet available - quality register 1114</t>
         </is>
       </c>
       <c r="L116" s="5" t="inlineStr">
@@ -7519,7 +7519,7 @@
       </c>
       <c r="K117" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1115</t>
+          <t>Pending - register map of the source device not yet available - quality register 1115</t>
         </is>
       </c>
       <c r="L117" s="5" t="inlineStr">
@@ -7575,7 +7575,7 @@
       </c>
       <c r="K118" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1116</t>
+          <t>Pending - register map of the source device not yet available - quality register 1116</t>
         </is>
       </c>
       <c r="L118" s="5" t="inlineStr">
@@ -7631,7 +7631,7 @@
       </c>
       <c r="K119" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1117</t>
+          <t>Pending - register map of the source device not yet available - quality register 1117</t>
         </is>
       </c>
       <c r="L119" s="5" t="inlineStr">
@@ -7687,7 +7687,7 @@
       </c>
       <c r="K120" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1118</t>
+          <t>Pending - register map of the source device not yet available - quality register 1118</t>
         </is>
       </c>
       <c r="L120" s="5" t="inlineStr">
@@ -7743,7 +7743,7 @@
       </c>
       <c r="K121" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1119</t>
+          <t>Pending - register map of the source device not yet available - quality register 1119</t>
         </is>
       </c>
       <c r="L121" s="5" t="inlineStr">
@@ -7799,7 +7799,7 @@
       </c>
       <c r="K122" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1120</t>
+          <t>Pending - register map of the source device not yet available - quality register 1120</t>
         </is>
       </c>
       <c r="L122" s="5" t="inlineStr">
@@ -7855,7 +7855,7 @@
       </c>
       <c r="K123" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1121</t>
+          <t>Pending - register map of the source device not yet available - quality register 1121</t>
         </is>
       </c>
       <c r="L123" s="5" t="inlineStr">
@@ -7911,7 +7911,7 @@
       </c>
       <c r="K124" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1122</t>
+          <t>Pending - register map of the source device not yet available - quality register 1122</t>
         </is>
       </c>
       <c r="L124" s="5" t="inlineStr">
@@ -7967,7 +7967,7 @@
       </c>
       <c r="K125" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1123</t>
+          <t>Pending - register map of the source device not yet available - quality register 1123</t>
         </is>
       </c>
       <c r="L125" s="5" t="inlineStr">
@@ -8023,7 +8023,7 @@
       </c>
       <c r="K126" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1124</t>
+          <t>Pending - register map of the source device not yet available - quality register 1124</t>
         </is>
       </c>
       <c r="L126" s="5" t="inlineStr">
@@ -8079,7 +8079,7 @@
       </c>
       <c r="K127" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1125</t>
+          <t>Pending - register map of the source device not yet available - quality register 1125</t>
         </is>
       </c>
       <c r="L127" s="5" t="inlineStr">
@@ -8131,7 +8131,7 @@
       </c>
       <c r="K128" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1126</t>
+          <t>Pending - register map of the source device not yet available - quality register 1126</t>
         </is>
       </c>
       <c r="L128" s="5" t="inlineStr">
@@ -8187,7 +8187,7 @@
       </c>
       <c r="K129" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1127</t>
+          <t>Pending - register map of the source device not yet available - quality register 1127</t>
         </is>
       </c>
       <c r="L129" s="5" t="inlineStr">
@@ -8243,7 +8243,7 @@
       </c>
       <c r="K130" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1128</t>
+          <t>Pending - register map of the source device not yet available - quality register 1128</t>
         </is>
       </c>
       <c r="L130" s="5" t="inlineStr">
@@ -8299,7 +8299,7 @@
       </c>
       <c r="K131" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1129</t>
+          <t>Pending - register map of the source device not yet available - quality register 1129</t>
         </is>
       </c>
       <c r="L131" s="5" t="inlineStr">
@@ -8355,7 +8355,7 @@
       </c>
       <c r="K132" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1130</t>
+          <t>Pending - register map of the source device not yet available - quality register 1130</t>
         </is>
       </c>
       <c r="L132" s="5" t="inlineStr">
@@ -8411,7 +8411,7 @@
       </c>
       <c r="K133" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1131</t>
+          <t>Pending - register map of the source device not yet available - quality register 1131</t>
         </is>
       </c>
       <c r="L133" s="5" t="inlineStr">
@@ -8467,7 +8467,7 @@
       </c>
       <c r="K134" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1132</t>
+          <t>Pending - register map of the source device not yet available - quality register 1132</t>
         </is>
       </c>
       <c r="L134" s="5" t="inlineStr">
@@ -8523,7 +8523,7 @@
       </c>
       <c r="K135" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1133</t>
+          <t>Pending - register map of the source device not yet available - quality register 1133</t>
         </is>
       </c>
       <c r="L135" s="5" t="inlineStr">
@@ -8579,7 +8579,7 @@
       </c>
       <c r="K136" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1134</t>
+          <t>Pending - register map of the source device not yet available - quality register 1134</t>
         </is>
       </c>
       <c r="L136" s="5" t="inlineStr">
@@ -8635,7 +8635,7 @@
       </c>
       <c r="K137" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1135</t>
+          <t>Pending - register map of the source device not yet available - quality register 1135</t>
         </is>
       </c>
       <c r="L137" s="5" t="inlineStr">
@@ -8691,7 +8691,7 @@
       </c>
       <c r="K138" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1136</t>
+          <t>Pending - register map of the source device not yet available - quality register 1136</t>
         </is>
       </c>
       <c r="L138" s="5" t="inlineStr">
@@ -8747,7 +8747,7 @@
       </c>
       <c r="K139" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1137</t>
+          <t>Pending - register map of the source device not yet available - quality register 1137</t>
         </is>
       </c>
       <c r="L139" s="5" t="inlineStr">
@@ -8803,7 +8803,7 @@
       </c>
       <c r="K140" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1138</t>
+          <t>Pending - register map of the source device not yet available - quality register 1138</t>
         </is>
       </c>
       <c r="L140" s="5" t="inlineStr">
@@ -8859,7 +8859,7 @@
       </c>
       <c r="K141" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1139</t>
+          <t>Pending - register map of the source device not yet available - quality register 1139</t>
         </is>
       </c>
       <c r="L141" s="5" t="inlineStr">
@@ -8915,7 +8915,7 @@
       </c>
       <c r="K142" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1140</t>
+          <t>Pending - register map of the source device not yet available - quality register 1140</t>
         </is>
       </c>
       <c r="L142" s="5" t="inlineStr">
@@ -8971,7 +8971,7 @@
       </c>
       <c r="K143" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1141</t>
+          <t>Pending - register map of the source device not yet available - quality register 1141</t>
         </is>
       </c>
       <c r="L143" s="5" t="inlineStr">
@@ -9027,7 +9027,7 @@
       </c>
       <c r="K144" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1142</t>
+          <t>Pending - register map of the source device not yet available - quality register 1142</t>
         </is>
       </c>
       <c r="L144" s="5" t="inlineStr">
@@ -9083,7 +9083,7 @@
       </c>
       <c r="K145" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1143</t>
+          <t>Pending - register map of the source device not yet available - quality register 1143</t>
         </is>
       </c>
       <c r="L145" s="5" t="inlineStr">
@@ -9139,7 +9139,7 @@
       </c>
       <c r="K146" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1144</t>
+          <t>Pending - register map of the source device not yet available - quality register 1144</t>
         </is>
       </c>
       <c r="L146" s="5" t="inlineStr">
@@ -9195,7 +9195,7 @@
       </c>
       <c r="K147" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1145</t>
+          <t>Pending - register map of the source device not yet available - quality register 1145</t>
         </is>
       </c>
       <c r="L147" s="5" t="inlineStr">
@@ -9251,7 +9251,7 @@
       </c>
       <c r="K148" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1146</t>
+          <t>Pending - register map of the source device not yet available - quality register 1146</t>
         </is>
       </c>
       <c r="L148" s="5" t="inlineStr">
@@ -9307,7 +9307,7 @@
       </c>
       <c r="K149" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1147</t>
+          <t>Pending - register map of the source device not yet available - quality register 1147</t>
         </is>
       </c>
       <c r="L149" s="5" t="inlineStr">
@@ -9363,7 +9363,7 @@
       </c>
       <c r="K150" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1148</t>
+          <t>Pending - register map of the source device not yet available - quality register 1148</t>
         </is>
       </c>
       <c r="L150" s="5" t="inlineStr">
@@ -9419,7 +9419,7 @@
       </c>
       <c r="K151" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1149</t>
+          <t>Pending - register map of the source device not yet available - quality register 1149</t>
         </is>
       </c>
       <c r="L151" s="5" t="inlineStr">
@@ -9475,7 +9475,7 @@
       </c>
       <c r="K152" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1150</t>
+          <t>Pending - register map of the source device not yet available - quality register 1150</t>
         </is>
       </c>
       <c r="L152" s="5" t="inlineStr">
@@ -9531,7 +9531,7 @@
       </c>
       <c r="K153" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1151</t>
+          <t>Pending - register map of the source device not yet available - quality register 1151</t>
         </is>
       </c>
       <c r="L153" s="5" t="inlineStr">
@@ -9587,7 +9587,7 @@
       </c>
       <c r="K154" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1152</t>
+          <t>Pending - register map of the source device not yet available - quality register 1152</t>
         </is>
       </c>
       <c r="L154" s="5" t="inlineStr">
@@ -9643,7 +9643,7 @@
       </c>
       <c r="K155" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1153</t>
+          <t>Pending - register map of the source device not yet available - quality register 1153</t>
         </is>
       </c>
       <c r="L155" s="5" t="inlineStr">
@@ -9699,7 +9699,7 @@
       </c>
       <c r="K156" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1154</t>
+          <t>Pending - register map of the source device not yet available - quality register 1154</t>
         </is>
       </c>
       <c r="L156" s="5" t="inlineStr">
@@ -9751,7 +9751,7 @@
       </c>
       <c r="K157" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1155</t>
+          <t>Pending - register map of the source device not yet available - quality register 1155</t>
         </is>
       </c>
       <c r="L157" s="5" t="inlineStr">
@@ -9807,7 +9807,7 @@
       </c>
       <c r="K158" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1156</t>
+          <t>Pending - register map of the source device not yet available - quality register 1156</t>
         </is>
       </c>
       <c r="L158" s="5" t="inlineStr">
@@ -9863,7 +9863,7 @@
       </c>
       <c r="K159" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1157</t>
+          <t>Pending - register map of the source device not yet available - quality register 1157</t>
         </is>
       </c>
       <c r="L159" s="5" t="inlineStr">
@@ -9919,7 +9919,7 @@
       </c>
       <c r="K160" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1158</t>
+          <t>Pending - register map of the source device not yet available - quality register 1158</t>
         </is>
       </c>
       <c r="L160" s="5" t="inlineStr">
@@ -9975,7 +9975,7 @@
       </c>
       <c r="K161" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1159</t>
+          <t>Pending - register map of the source device not yet available - quality register 1159</t>
         </is>
       </c>
       <c r="L161" s="5" t="inlineStr">
@@ -10031,7 +10031,7 @@
       </c>
       <c r="K162" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1160</t>
+          <t>Pending - register map of the source device not yet available - quality register 1160</t>
         </is>
       </c>
       <c r="L162" s="5" t="inlineStr">
@@ -10087,7 +10087,7 @@
       </c>
       <c r="K163" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1161</t>
+          <t>Pending - register map of the source device not yet available - quality register 1161</t>
         </is>
       </c>
       <c r="L163" s="5" t="inlineStr">
@@ -10143,7 +10143,7 @@
       </c>
       <c r="K164" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1162</t>
+          <t>Pending - register map of the source device not yet available - quality register 1162</t>
         </is>
       </c>
       <c r="L164" s="5" t="inlineStr">
@@ -10199,7 +10199,7 @@
       </c>
       <c r="K165" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1163</t>
+          <t>Pending - register map of the source device not yet available - quality register 1163</t>
         </is>
       </c>
       <c r="L165" s="5" t="inlineStr">
@@ -10255,7 +10255,7 @@
       </c>
       <c r="K166" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1164</t>
+          <t>Pending - register map of the source device not yet available - quality register 1164</t>
         </is>
       </c>
       <c r="L166" s="5" t="inlineStr">
@@ -10311,7 +10311,7 @@
       </c>
       <c r="K167" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1165</t>
+          <t>Pending - register map of the source device not yet available - quality register 1165</t>
         </is>
       </c>
       <c r="L167" s="5" t="inlineStr">
@@ -10367,7 +10367,7 @@
       </c>
       <c r="K168" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1166</t>
+          <t>Pending - register map of the source device not yet available - quality register 1166</t>
         </is>
       </c>
       <c r="L168" s="5" t="inlineStr">
@@ -10423,7 +10423,7 @@
       </c>
       <c r="K169" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1167</t>
+          <t>Pending - register map of the source device not yet available - quality register 1167</t>
         </is>
       </c>
       <c r="L169" s="5" t="inlineStr">
@@ -10479,7 +10479,7 @@
       </c>
       <c r="K170" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1168</t>
+          <t>Pending - register map of the source device not yet available - quality register 1168</t>
         </is>
       </c>
       <c r="L170" s="5" t="inlineStr">
@@ -10535,7 +10535,7 @@
       </c>
       <c r="K171" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1169</t>
+          <t>Pending - register map of the source device not yet available - quality register 1169</t>
         </is>
       </c>
       <c r="L171" s="5" t="inlineStr">
@@ -10591,7 +10591,7 @@
       </c>
       <c r="K172" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1170</t>
+          <t>Pending - register map of the source device not yet available - quality register 1170</t>
         </is>
       </c>
       <c r="L172" s="5" t="inlineStr">
@@ -10647,7 +10647,7 @@
       </c>
       <c r="K173" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1171</t>
+          <t>Pending - register map of the source device not yet available - quality register 1171</t>
         </is>
       </c>
       <c r="L173" s="5" t="inlineStr">
@@ -10703,7 +10703,7 @@
       </c>
       <c r="K174" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1172</t>
+          <t>Pending - register map of the source device not yet available - quality register 1172</t>
         </is>
       </c>
       <c r="L174" s="5" t="inlineStr">
@@ -10759,7 +10759,7 @@
       </c>
       <c r="K175" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1173</t>
+          <t>Pending - register map of the source device not yet available - quality register 1173</t>
         </is>
       </c>
       <c r="L175" s="5" t="inlineStr">
@@ -10815,7 +10815,7 @@
       </c>
       <c r="K176" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1174</t>
+          <t>Pending - register map of the source device not yet available - quality register 1174</t>
         </is>
       </c>
       <c r="L176" s="5" t="inlineStr">
@@ -10871,7 +10871,7 @@
       </c>
       <c r="K177" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1175</t>
+          <t>Pending - register map of the source device not yet available - quality register 1175</t>
         </is>
       </c>
       <c r="L177" s="5" t="inlineStr">
@@ -10927,7 +10927,7 @@
       </c>
       <c r="K178" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1176</t>
+          <t>Pending - register map of the source device not yet available - quality register 1176</t>
         </is>
       </c>
       <c r="L178" s="5" t="inlineStr">
@@ -10983,7 +10983,7 @@
       </c>
       <c r="K179" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1177</t>
+          <t>Pending - register map of the source device not yet available - quality register 1177</t>
         </is>
       </c>
       <c r="L179" s="5" t="inlineStr">
@@ -11039,7 +11039,7 @@
       </c>
       <c r="K180" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1178</t>
+          <t>Pending - register map of the source device not yet available - quality register 1178</t>
         </is>
       </c>
       <c r="L180" s="5" t="inlineStr">
@@ -11095,7 +11095,7 @@
       </c>
       <c r="K181" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1179</t>
+          <t>Pending - register map of the source device not yet available - quality register 1179</t>
         </is>
       </c>
       <c r="L181" s="5" t="inlineStr">
@@ -11151,7 +11151,7 @@
       </c>
       <c r="K182" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1180</t>
+          <t>Pending - register map of the source device not yet available - quality register 1180</t>
         </is>
       </c>
       <c r="L182" s="5" t="inlineStr">
@@ -11207,7 +11207,7 @@
       </c>
       <c r="K183" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1181</t>
+          <t>Pending - register map of the source device not yet available - quality register 1181</t>
         </is>
       </c>
       <c r="L183" s="5" t="inlineStr">
@@ -11263,7 +11263,7 @@
       </c>
       <c r="K184" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1182</t>
+          <t>Pending - register map of the source device not yet available - quality register 1182</t>
         </is>
       </c>
       <c r="L184" s="5" t="inlineStr">
@@ -11319,7 +11319,7 @@
       </c>
       <c r="K185" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1183</t>
+          <t>Pending - register map of the source device not yet available - quality register 1183</t>
         </is>
       </c>
       <c r="L185" s="5" t="inlineStr">
@@ -11371,7 +11371,7 @@
       </c>
       <c r="K186" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1184</t>
+          <t>Pending - register map of the source device not yet available - quality register 1184</t>
         </is>
       </c>
       <c r="L186" s="5" t="inlineStr">
@@ -11427,7 +11427,7 @@
       </c>
       <c r="K187" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1185</t>
+          <t>Pending - register map of the source device not yet available - quality register 1185</t>
         </is>
       </c>
       <c r="L187" s="5" t="inlineStr">
@@ -11483,7 +11483,7 @@
       </c>
       <c r="K188" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1186</t>
+          <t>Pending - register map of the source device not yet available - quality register 1186</t>
         </is>
       </c>
       <c r="L188" s="5" t="inlineStr">
@@ -11539,7 +11539,7 @@
       </c>
       <c r="K189" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1187</t>
+          <t>Pending - register map of the source device not yet available - quality register 1187</t>
         </is>
       </c>
       <c r="L189" s="5" t="inlineStr">
@@ -11595,7 +11595,7 @@
       </c>
       <c r="K190" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1188</t>
+          <t>Pending - register map of the source device not yet available - quality register 1188</t>
         </is>
       </c>
       <c r="L190" s="5" t="inlineStr">
@@ -11651,7 +11651,7 @@
       </c>
       <c r="K191" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1189</t>
+          <t>Pending - register map of the source device not yet available - quality register 1189</t>
         </is>
       </c>
       <c r="L191" s="5" t="inlineStr">
@@ -11707,7 +11707,7 @@
       </c>
       <c r="K192" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1190</t>
+          <t>Pending - register map of the source device not yet available - quality register 1190</t>
         </is>
       </c>
       <c r="L192" s="5" t="inlineStr">
@@ -11763,7 +11763,7 @@
       </c>
       <c r="K193" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1191</t>
+          <t>Pending - register map of the source device not yet available - quality register 1191</t>
         </is>
       </c>
       <c r="L193" s="5" t="inlineStr">
@@ -11819,7 +11819,7 @@
       </c>
       <c r="K194" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1192</t>
+          <t>Pending - register map of the source device not yet available - quality register 1192</t>
         </is>
       </c>
       <c r="L194" s="5" t="inlineStr">
@@ -11875,7 +11875,7 @@
       </c>
       <c r="K195" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1193</t>
+          <t>Pending - register map of the source device not yet available - quality register 1193</t>
         </is>
       </c>
       <c r="L195" s="5" t="inlineStr">
@@ -11931,7 +11931,7 @@
       </c>
       <c r="K196" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1194</t>
+          <t>Pending - register map of the source device not yet available - quality register 1194</t>
         </is>
       </c>
       <c r="L196" s="5" t="inlineStr">
@@ -11987,7 +11987,7 @@
       </c>
       <c r="K197" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1195</t>
+          <t>Pending - register map of the source device not yet available - quality register 1195</t>
         </is>
       </c>
       <c r="L197" s="5" t="inlineStr">
@@ -12043,7 +12043,7 @@
       </c>
       <c r="K198" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1196</t>
+          <t>Pending - register map of the source device not yet available - quality register 1196</t>
         </is>
       </c>
       <c r="L198" s="5" t="inlineStr">
@@ -12099,7 +12099,7 @@
       </c>
       <c r="K199" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1197</t>
+          <t>Pending - register map of the source device not yet available - quality register 1197</t>
         </is>
       </c>
       <c r="L199" s="5" t="inlineStr">
@@ -12155,7 +12155,7 @@
       </c>
       <c r="K200" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1198</t>
+          <t>Pending - register map of the source device not yet available - quality register 1198</t>
         </is>
       </c>
       <c r="L200" s="5" t="inlineStr">
@@ -12211,7 +12211,7 @@
       </c>
       <c r="K201" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1199</t>
+          <t>Pending - register map of the source device not yet available - quality register 1199</t>
         </is>
       </c>
       <c r="L201" s="5" t="inlineStr">
@@ -12267,7 +12267,7 @@
       </c>
       <c r="K202" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1200</t>
+          <t>Pending - register map of the source device not yet available - quality register 1200</t>
         </is>
       </c>
       <c r="L202" s="5" t="inlineStr">
@@ -12323,7 +12323,7 @@
       </c>
       <c r="K203" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1201</t>
+          <t>Pending - register map of the source device not yet available - quality register 1201</t>
         </is>
       </c>
       <c r="L203" s="5" t="inlineStr">
@@ -12379,7 +12379,7 @@
       </c>
       <c r="K204" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1202</t>
+          <t>Pending - register map of the source device not yet available - quality register 1202</t>
         </is>
       </c>
       <c r="L204" s="5" t="inlineStr">
@@ -12435,7 +12435,7 @@
       </c>
       <c r="K205" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1203</t>
+          <t>Pending - register map of the source device not yet available - quality register 1203</t>
         </is>
       </c>
       <c r="L205" s="5" t="inlineStr">
@@ -12491,7 +12491,7 @@
       </c>
       <c r="K206" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1204</t>
+          <t>Pending - register map of the source device not yet available - quality register 1204</t>
         </is>
       </c>
       <c r="L206" s="5" t="inlineStr">
@@ -12547,7 +12547,7 @@
       </c>
       <c r="K207" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1205</t>
+          <t>Pending - register map of the source device not yet available - quality register 1205</t>
         </is>
       </c>
       <c r="L207" s="5" t="inlineStr">
@@ -12603,7 +12603,7 @@
       </c>
       <c r="K208" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1206</t>
+          <t>Pending - register map of the source device not yet available - quality register 1206</t>
         </is>
       </c>
       <c r="L208" s="5" t="inlineStr">
@@ -12659,7 +12659,7 @@
       </c>
       <c r="K209" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1207</t>
+          <t>Pending - register map of the source device not yet available - quality register 1207</t>
         </is>
       </c>
       <c r="L209" s="5" t="inlineStr">
@@ -12715,7 +12715,7 @@
       </c>
       <c r="K210" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1208</t>
+          <t>Pending - register map of the source device not yet available - quality register 1208</t>
         </is>
       </c>
       <c r="L210" s="5" t="inlineStr">
@@ -12771,7 +12771,7 @@
       </c>
       <c r="K211" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1209</t>
+          <t>Pending - register map of the source device not yet available - quality register 1209</t>
         </is>
       </c>
       <c r="L211" s="5" t="inlineStr">
@@ -12827,7 +12827,7 @@
       </c>
       <c r="K212" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1210</t>
+          <t>Pending - register map of the source device not yet available - quality register 1210</t>
         </is>
       </c>
       <c r="L212" s="5" t="inlineStr">
@@ -12883,7 +12883,7 @@
       </c>
       <c r="K213" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1211</t>
+          <t>Pending - register map of the source device not yet available - quality register 1211</t>
         </is>
       </c>
       <c r="L213" s="5" t="inlineStr">
@@ -12939,7 +12939,7 @@
       </c>
       <c r="K214" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1212</t>
+          <t>Pending - register map of the source device not yet available - quality register 1212</t>
         </is>
       </c>
       <c r="L214" s="5" t="inlineStr">
@@ -12991,7 +12991,7 @@
       </c>
       <c r="K215" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1213</t>
+          <t>Pending - register map of the source device not yet available - quality register 1213</t>
         </is>
       </c>
       <c r="L215" s="5" t="inlineStr">
@@ -13047,7 +13047,7 @@
       </c>
       <c r="K216" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1214</t>
+          <t>Pending - register map of the source device not yet available - quality register 1214</t>
         </is>
       </c>
       <c r="L216" s="5" t="inlineStr">
@@ -13103,7 +13103,7 @@
       </c>
       <c r="K217" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1215</t>
+          <t>Pending - register map of the source device not yet available - quality register 1215</t>
         </is>
       </c>
       <c r="L217" s="5" t="inlineStr">
@@ -13159,7 +13159,7 @@
       </c>
       <c r="K218" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1216</t>
+          <t>Pending - register map of the source device not yet available - quality register 1216</t>
         </is>
       </c>
       <c r="L218" s="5" t="inlineStr">
@@ -13215,7 +13215,7 @@
       </c>
       <c r="K219" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1217</t>
+          <t>Pending - register map of the source device not yet available - quality register 1217</t>
         </is>
       </c>
       <c r="L219" s="5" t="inlineStr">
@@ -13271,7 +13271,7 @@
       </c>
       <c r="K220" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1218</t>
+          <t>Pending - register map of the source device not yet available - quality register 1218</t>
         </is>
       </c>
       <c r="L220" s="5" t="inlineStr">
@@ -13327,7 +13327,7 @@
       </c>
       <c r="K221" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1219</t>
+          <t>Pending - register map of the source device not yet available - quality register 1219</t>
         </is>
       </c>
       <c r="L221" s="5" t="inlineStr">
@@ -13383,7 +13383,7 @@
       </c>
       <c r="K222" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1220</t>
+          <t>Pending - register map of the source device not yet available - quality register 1220</t>
         </is>
       </c>
       <c r="L222" s="5" t="inlineStr">
@@ -13439,7 +13439,7 @@
       </c>
       <c r="K223" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1221</t>
+          <t>Pending - register map of the source device not yet available - quality register 1221</t>
         </is>
       </c>
       <c r="L223" s="5" t="inlineStr">
@@ -13495,7 +13495,7 @@
       </c>
       <c r="K224" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1222</t>
+          <t>Pending - register map of the source device not yet available - quality register 1222</t>
         </is>
       </c>
       <c r="L224" s="5" t="inlineStr">
@@ -13551,7 +13551,7 @@
       </c>
       <c r="K225" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1223</t>
+          <t>Pending - register map of the source device not yet available - quality register 1223</t>
         </is>
       </c>
       <c r="L225" s="5" t="inlineStr">
@@ -13607,7 +13607,7 @@
       </c>
       <c r="K226" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1224</t>
+          <t>Pending - register map of the source device not yet available - quality register 1224</t>
         </is>
       </c>
       <c r="L226" s="5" t="inlineStr">
@@ -13663,7 +13663,7 @@
       </c>
       <c r="K227" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1225</t>
+          <t>Pending - register map of the source device not yet available - quality register 1225</t>
         </is>
       </c>
       <c r="L227" s="5" t="inlineStr">
@@ -13719,7 +13719,7 @@
       </c>
       <c r="K228" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1226</t>
+          <t>Pending - register map of the source device not yet available - quality register 1226</t>
         </is>
       </c>
       <c r="L228" s="5" t="inlineStr">
@@ -13775,7 +13775,7 @@
       </c>
       <c r="K229" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1227</t>
+          <t>Pending - register map of the source device not yet available - quality register 1227</t>
         </is>
       </c>
       <c r="L229" s="5" t="inlineStr">
@@ -13831,7 +13831,7 @@
       </c>
       <c r="K230" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1228</t>
+          <t>Pending - register map of the source device not yet available - quality register 1228</t>
         </is>
       </c>
       <c r="L230" s="5" t="inlineStr">
@@ -13887,7 +13887,7 @@
       </c>
       <c r="K231" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1229</t>
+          <t>Pending - register map of the source device not yet available - quality register 1229</t>
         </is>
       </c>
       <c r="L231" s="5" t="inlineStr">
@@ -13943,7 +13943,7 @@
       </c>
       <c r="K232" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1230</t>
+          <t>Pending - register map of the source device not yet available - quality register 1230</t>
         </is>
       </c>
       <c r="L232" s="5" t="inlineStr">
@@ -13999,7 +13999,7 @@
       </c>
       <c r="K233" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1231</t>
+          <t>Pending - register map of the source device not yet available - quality register 1231</t>
         </is>
       </c>
       <c r="L233" s="5" t="inlineStr">
@@ -14055,7 +14055,7 @@
       </c>
       <c r="K234" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1232</t>
+          <t>Pending - register map of the source device not yet available - quality register 1232</t>
         </is>
       </c>
       <c r="L234" s="5" t="inlineStr">
@@ -14111,7 +14111,7 @@
       </c>
       <c r="K235" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1233</t>
+          <t>Pending - register map of the source device not yet available - quality register 1233</t>
         </is>
       </c>
       <c r="L235" s="5" t="inlineStr">
@@ -14167,7 +14167,7 @@
       </c>
       <c r="K236" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1234</t>
+          <t>Pending - register map of the source device not yet available - quality register 1234</t>
         </is>
       </c>
       <c r="L236" s="5" t="inlineStr">
@@ -14223,7 +14223,7 @@
       </c>
       <c r="K237" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1235</t>
+          <t>Pending - register map of the source device not yet available - quality register 1235</t>
         </is>
       </c>
       <c r="L237" s="5" t="inlineStr">
@@ -14279,7 +14279,7 @@
       </c>
       <c r="K238" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1236</t>
+          <t>Pending - register map of the source device not yet available - quality register 1236</t>
         </is>
       </c>
       <c r="L238" s="5" t="inlineStr">
@@ -14335,7 +14335,7 @@
       </c>
       <c r="K239" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1237</t>
+          <t>Pending - register map of the source device not yet available - quality register 1237</t>
         </is>
       </c>
       <c r="L239" s="5" t="inlineStr">
@@ -14391,7 +14391,7 @@
       </c>
       <c r="K240" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1238</t>
+          <t>Pending - register map of the source device not yet available - quality register 1238</t>
         </is>
       </c>
       <c r="L240" s="5" t="inlineStr">
@@ -14447,7 +14447,7 @@
       </c>
       <c r="K241" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1239</t>
+          <t>Pending - register map of the source device not yet available - quality register 1239</t>
         </is>
       </c>
       <c r="L241" s="5" t="inlineStr">
@@ -14503,7 +14503,7 @@
       </c>
       <c r="K242" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1240</t>
+          <t>Pending - register map of the source device not yet available - quality register 1240</t>
         </is>
       </c>
       <c r="L242" s="5" t="inlineStr">
@@ -14559,7 +14559,7 @@
       </c>
       <c r="K243" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1241</t>
+          <t>Pending - register map of the source device not yet available - quality register 1241</t>
         </is>
       </c>
       <c r="L243" s="5" t="inlineStr">
@@ -14611,7 +14611,7 @@
       </c>
       <c r="K244" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1242</t>
+          <t>Pending - register map of the source device not yet available - quality register 1242</t>
         </is>
       </c>
       <c r="L244" s="5" t="inlineStr">
@@ -14667,7 +14667,7 @@
       </c>
       <c r="K245" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1243</t>
+          <t>Pending - register map of the source device not yet available - quality register 1243</t>
         </is>
       </c>
       <c r="L245" s="5" t="inlineStr">
@@ -14723,7 +14723,7 @@
       </c>
       <c r="K246" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1244</t>
+          <t>Pending - register map of the source device not yet available - quality register 1244</t>
         </is>
       </c>
       <c r="L246" s="5" t="inlineStr">
@@ -14779,7 +14779,7 @@
       </c>
       <c r="K247" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1245</t>
+          <t>Pending - register map of the source device not yet available - quality register 1245</t>
         </is>
       </c>
       <c r="L247" s="5" t="inlineStr">
@@ -14835,7 +14835,7 @@
       </c>
       <c r="K248" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1246</t>
+          <t>Pending - register map of the source device not yet available - quality register 1246</t>
         </is>
       </c>
       <c r="L248" s="5" t="inlineStr">
@@ -14891,7 +14891,7 @@
       </c>
       <c r="K249" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1247</t>
+          <t>Pending - register map of the source device not yet available - quality register 1247</t>
         </is>
       </c>
       <c r="L249" s="5" t="inlineStr">
@@ -14947,7 +14947,7 @@
       </c>
       <c r="K250" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1248</t>
+          <t>Pending - register map of the source device not yet available - quality register 1248</t>
         </is>
       </c>
       <c r="L250" s="5" t="inlineStr">
@@ -15003,7 +15003,7 @@
       </c>
       <c r="K251" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1249</t>
+          <t>Pending - register map of the source device not yet available - quality register 1249</t>
         </is>
       </c>
       <c r="L251" s="5" t="inlineStr">
@@ -15059,7 +15059,7 @@
       </c>
       <c r="K252" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1250</t>
+          <t>Pending - register map of the source device not yet available - quality register 1250</t>
         </is>
       </c>
       <c r="L252" s="5" t="inlineStr">
@@ -15115,7 +15115,7 @@
       </c>
       <c r="K253" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1251</t>
+          <t>Pending - register map of the source device not yet available - quality register 1251</t>
         </is>
       </c>
       <c r="L253" s="5" t="inlineStr">
@@ -15171,7 +15171,7 @@
       </c>
       <c r="K254" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1252</t>
+          <t>Pending - register map of the source device not yet available - quality register 1252</t>
         </is>
       </c>
       <c r="L254" s="5" t="inlineStr">
@@ -15227,7 +15227,7 @@
       </c>
       <c r="K255" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1253</t>
+          <t>Pending - register map of the source device not yet available - quality register 1253</t>
         </is>
       </c>
       <c r="L255" s="5" t="inlineStr">
@@ -15283,7 +15283,7 @@
       </c>
       <c r="K256" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1254</t>
+          <t>Pending - register map of the source device not yet available - quality register 1254</t>
         </is>
       </c>
       <c r="L256" s="5" t="inlineStr">
@@ -15339,7 +15339,7 @@
       </c>
       <c r="K257" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1255</t>
+          <t>Pending - register map of the source device not yet available - quality register 1255</t>
         </is>
       </c>
       <c r="L257" s="5" t="inlineStr">
@@ -15395,7 +15395,7 @@
       </c>
       <c r="K258" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1256</t>
+          <t>Pending - register map of the source device not yet available - quality register 1256</t>
         </is>
       </c>
       <c r="L258" s="5" t="inlineStr">
@@ -15451,7 +15451,7 @@
       </c>
       <c r="K259" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1257</t>
+          <t>Pending - register map of the source device not yet available - quality register 1257</t>
         </is>
       </c>
       <c r="L259" s="5" t="inlineStr">
@@ -15507,7 +15507,7 @@
       </c>
       <c r="K260" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1258</t>
+          <t>Pending - register map of the source device not yet available - quality register 1258</t>
         </is>
       </c>
       <c r="L260" s="5" t="inlineStr">
@@ -15563,7 +15563,7 @@
       </c>
       <c r="K261" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1259</t>
+          <t>Pending - register map of the source device not yet available - quality register 1259</t>
         </is>
       </c>
       <c r="L261" s="5" t="inlineStr">
@@ -15619,7 +15619,7 @@
       </c>
       <c r="K262" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1260</t>
+          <t>Pending - register map of the source device not yet available - quality register 1260</t>
         </is>
       </c>
       <c r="L262" s="5" t="inlineStr">
@@ -15675,7 +15675,7 @@
       </c>
       <c r="K263" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1261</t>
+          <t>Pending - register map of the source device not yet available - quality register 1261</t>
         </is>
       </c>
       <c r="L263" s="5" t="inlineStr">
@@ -15731,7 +15731,7 @@
       </c>
       <c r="K264" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1262</t>
+          <t>Pending - register map of the source device not yet available - quality register 1262</t>
         </is>
       </c>
       <c r="L264" s="5" t="inlineStr">
@@ -15787,7 +15787,7 @@
       </c>
       <c r="K265" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1263</t>
+          <t>Pending - register map of the source device not yet available - quality register 1263</t>
         </is>
       </c>
       <c r="L265" s="5" t="inlineStr">
@@ -15843,7 +15843,7 @@
       </c>
       <c r="K266" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1264</t>
+          <t>Pending - register map of the source device not yet available - quality register 1264</t>
         </is>
       </c>
       <c r="L266" s="5" t="inlineStr">
@@ -15899,7 +15899,7 @@
       </c>
       <c r="K267" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1265</t>
+          <t>Pending - register map of the source device not yet available - quality register 1265</t>
         </is>
       </c>
       <c r="L267" s="5" t="inlineStr">
@@ -15955,7 +15955,7 @@
       </c>
       <c r="K268" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1266</t>
+          <t>Pending - register map of the source device not yet available - quality register 1266</t>
         </is>
       </c>
       <c r="L268" s="5" t="inlineStr">
@@ -16011,7 +16011,7 @@
       </c>
       <c r="K269" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1267</t>
+          <t>Pending - register map of the source device not yet available - quality register 1267</t>
         </is>
       </c>
       <c r="L269" s="5" t="inlineStr">
@@ -16067,7 +16067,7 @@
       </c>
       <c r="K270" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1268</t>
+          <t>Pending - register map of the source device not yet available - quality register 1268</t>
         </is>
       </c>
       <c r="L270" s="5" t="inlineStr">
@@ -16123,7 +16123,7 @@
       </c>
       <c r="K271" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1269</t>
+          <t>Pending - register map of the source device not yet available - quality register 1269</t>
         </is>
       </c>
       <c r="L271" s="5" t="inlineStr">
@@ -16179,7 +16179,7 @@
       </c>
       <c r="K272" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1270</t>
+          <t>Pending - register map of the source device not yet available - quality register 1270</t>
         </is>
       </c>
       <c r="L272" s="5" t="inlineStr">
@@ -16231,7 +16231,7 @@
       </c>
       <c r="K273" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1271</t>
+          <t>Pending - register map of the source device not yet available - quality register 1271</t>
         </is>
       </c>
       <c r="L273" s="5" t="inlineStr">
@@ -16287,7 +16287,7 @@
       </c>
       <c r="K274" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1272</t>
+          <t>Pending - register map of the source device not yet available - quality register 1272</t>
         </is>
       </c>
       <c r="L274" s="5" t="inlineStr">
@@ -16343,7 +16343,7 @@
       </c>
       <c r="K275" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1273</t>
+          <t>Pending - register map of the source device not yet available - quality register 1273</t>
         </is>
       </c>
       <c r="L275" s="5" t="inlineStr">
@@ -16399,7 +16399,7 @@
       </c>
       <c r="K276" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1274</t>
+          <t>Pending - register map of the source device not yet available - quality register 1274</t>
         </is>
       </c>
       <c r="L276" s="5" t="inlineStr">
@@ -16455,7 +16455,7 @@
       </c>
       <c r="K277" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1275</t>
+          <t>Pending - register map of the source device not yet available - quality register 1275</t>
         </is>
       </c>
       <c r="L277" s="5" t="inlineStr">
@@ -16511,7 +16511,7 @@
       </c>
       <c r="K278" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1276</t>
+          <t>Pending - register map of the source device not yet available - quality register 1276</t>
         </is>
       </c>
       <c r="L278" s="5" t="inlineStr">
@@ -16567,7 +16567,7 @@
       </c>
       <c r="K279" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1277</t>
+          <t>Pending - register map of the source device not yet available - quality register 1277</t>
         </is>
       </c>
       <c r="L279" s="5" t="inlineStr">
@@ -16623,7 +16623,7 @@
       </c>
       <c r="K280" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1278</t>
+          <t>Pending - register map of the source device not yet available - quality register 1278</t>
         </is>
       </c>
       <c r="L280" s="5" t="inlineStr">
@@ -16679,7 +16679,7 @@
       </c>
       <c r="K281" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1279</t>
+          <t>Pending - register map of the source device not yet available - quality register 1279</t>
         </is>
       </c>
       <c r="L281" s="5" t="inlineStr">
@@ -16735,7 +16735,7 @@
       </c>
       <c r="K282" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1280</t>
+          <t>Pending - register map of the source device not yet available - quality register 1280</t>
         </is>
       </c>
       <c r="L282" s="5" t="inlineStr">
@@ -16791,7 +16791,7 @@
       </c>
       <c r="K283" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1281</t>
+          <t>Pending - register map of the source device not yet available - quality register 1281</t>
         </is>
       </c>
       <c r="L283" s="5" t="inlineStr">
@@ -16847,7 +16847,7 @@
       </c>
       <c r="K284" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1282</t>
+          <t>Pending - register map of the source device not yet available - quality register 1282</t>
         </is>
       </c>
       <c r="L284" s="5" t="inlineStr">
@@ -16903,7 +16903,7 @@
       </c>
       <c r="K285" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1283</t>
+          <t>Pending - register map of the source device not yet available - quality register 1283</t>
         </is>
       </c>
       <c r="L285" s="5" t="inlineStr">
@@ -16959,7 +16959,7 @@
       </c>
       <c r="K286" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1284</t>
+          <t>Pending - register map of the source device not yet available - quality register 1284</t>
         </is>
       </c>
       <c r="L286" s="5" t="inlineStr">
@@ -17015,7 +17015,7 @@
       </c>
       <c r="K287" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1285</t>
+          <t>Pending - register map of the source device not yet available - quality register 1285</t>
         </is>
       </c>
       <c r="L287" s="5" t="inlineStr">
@@ -17071,7 +17071,7 @@
       </c>
       <c r="K288" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1286</t>
+          <t>Pending - register map of the source device not yet available - quality register 1286</t>
         </is>
       </c>
       <c r="L288" s="5" t="inlineStr">
@@ -17127,7 +17127,7 @@
       </c>
       <c r="K289" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1287</t>
+          <t>Pending - register map of the source device not yet available - quality register 1287</t>
         </is>
       </c>
       <c r="L289" s="5" t="inlineStr">
@@ -17183,7 +17183,7 @@
       </c>
       <c r="K290" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1288</t>
+          <t>Pending - register map of the source device not yet available - quality register 1288</t>
         </is>
       </c>
       <c r="L290" s="5" t="inlineStr">
@@ -17239,7 +17239,7 @@
       </c>
       <c r="K291" s="6" t="inlineStr">
         <is>
-          <t>Ready — quality register 1289</t>
+          <t>Pending - register map of the source device not yet available - quality register 1289</t>
         </is>
       </c>
       <c r="L291" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Turkey workbooks: neutral commissioning status wording
</commit_message>
<xml_diff>
--- a/docs/turkey/Solar_Inverter_Tag_List_Rev.1.2.xlsx
+++ b/docs/turkey/Solar_Inverter_Tag_List_Rev.1.2.xlsx
@@ -1095,7 +1095,7 @@
       </c>
       <c r="K2" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1000</t>
+          <t>Pending commissioning - quality register 1000</t>
         </is>
       </c>
       <c r="L2" s="5" t="inlineStr">
@@ -1151,7 +1151,7 @@
       </c>
       <c r="K3" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1001</t>
+          <t>Pending commissioning - quality register 1001</t>
         </is>
       </c>
       <c r="L3" s="5" t="inlineStr">
@@ -1207,7 +1207,7 @@
       </c>
       <c r="K4" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1002</t>
+          <t>Pending commissioning - quality register 1002</t>
         </is>
       </c>
       <c r="L4" s="5" t="inlineStr">
@@ -1263,7 +1263,7 @@
       </c>
       <c r="K5" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1003</t>
+          <t>Pending commissioning - quality register 1003</t>
         </is>
       </c>
       <c r="L5" s="5" t="inlineStr">
@@ -1319,7 +1319,7 @@
       </c>
       <c r="K6" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1004</t>
+          <t>Pending commissioning - quality register 1004</t>
         </is>
       </c>
       <c r="L6" s="5" t="inlineStr">
@@ -1375,7 +1375,7 @@
       </c>
       <c r="K7" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1005</t>
+          <t>Pending commissioning - quality register 1005</t>
         </is>
       </c>
       <c r="L7" s="5" t="inlineStr">
@@ -1431,7 +1431,7 @@
       </c>
       <c r="K8" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1006</t>
+          <t>Pending commissioning - quality register 1006</t>
         </is>
       </c>
       <c r="L8" s="5" t="inlineStr">
@@ -1487,7 +1487,7 @@
       </c>
       <c r="K9" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1007</t>
+          <t>Pending commissioning - quality register 1007</t>
         </is>
       </c>
       <c r="L9" s="5" t="inlineStr">
@@ -1543,7 +1543,7 @@
       </c>
       <c r="K10" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1008</t>
+          <t>Pending commissioning - quality register 1008</t>
         </is>
       </c>
       <c r="L10" s="5" t="inlineStr">
@@ -1599,7 +1599,7 @@
       </c>
       <c r="K11" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1009</t>
+          <t>Pending commissioning - quality register 1009</t>
         </is>
       </c>
       <c r="L11" s="5" t="inlineStr">
@@ -1651,7 +1651,7 @@
       </c>
       <c r="K12" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1010</t>
+          <t>Pending commissioning - quality register 1010</t>
         </is>
       </c>
       <c r="L12" s="5" t="inlineStr">
@@ -1707,7 +1707,7 @@
       </c>
       <c r="K13" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1011</t>
+          <t>Pending commissioning - quality register 1011</t>
         </is>
       </c>
       <c r="L13" s="5" t="inlineStr">
@@ -1763,7 +1763,7 @@
       </c>
       <c r="K14" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1012</t>
+          <t>Pending commissioning - quality register 1012</t>
         </is>
       </c>
       <c r="L14" s="5" t="inlineStr">
@@ -1819,7 +1819,7 @@
       </c>
       <c r="K15" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1013</t>
+          <t>Pending commissioning - quality register 1013</t>
         </is>
       </c>
       <c r="L15" s="5" t="inlineStr">
@@ -1875,7 +1875,7 @@
       </c>
       <c r="K16" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1014</t>
+          <t>Pending commissioning - quality register 1014</t>
         </is>
       </c>
       <c r="L16" s="5" t="inlineStr">
@@ -1931,7 +1931,7 @@
       </c>
       <c r="K17" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1015</t>
+          <t>Pending commissioning - quality register 1015</t>
         </is>
       </c>
       <c r="L17" s="5" t="inlineStr">
@@ -1987,7 +1987,7 @@
       </c>
       <c r="K18" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1016</t>
+          <t>Pending commissioning - quality register 1016</t>
         </is>
       </c>
       <c r="L18" s="5" t="inlineStr">
@@ -2043,7 +2043,7 @@
       </c>
       <c r="K19" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1017</t>
+          <t>Pending commissioning - quality register 1017</t>
         </is>
       </c>
       <c r="L19" s="5" t="inlineStr">
@@ -2099,7 +2099,7 @@
       </c>
       <c r="K20" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1018</t>
+          <t>Pending commissioning - quality register 1018</t>
         </is>
       </c>
       <c r="L20" s="5" t="inlineStr">
@@ -2155,7 +2155,7 @@
       </c>
       <c r="K21" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1019</t>
+          <t>Pending commissioning - quality register 1019</t>
         </is>
       </c>
       <c r="L21" s="5" t="inlineStr">
@@ -2211,7 +2211,7 @@
       </c>
       <c r="K22" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1020</t>
+          <t>Pending commissioning - quality register 1020</t>
         </is>
       </c>
       <c r="L22" s="5" t="inlineStr">
@@ -2267,7 +2267,7 @@
       </c>
       <c r="K23" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1021</t>
+          <t>Pending commissioning - quality register 1021</t>
         </is>
       </c>
       <c r="L23" s="5" t="inlineStr">
@@ -2323,7 +2323,7 @@
       </c>
       <c r="K24" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1022</t>
+          <t>Pending commissioning - quality register 1022</t>
         </is>
       </c>
       <c r="L24" s="5" t="inlineStr">
@@ -2379,7 +2379,7 @@
       </c>
       <c r="K25" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1023</t>
+          <t>Pending commissioning - quality register 1023</t>
         </is>
       </c>
       <c r="L25" s="5" t="inlineStr">
@@ -2435,7 +2435,7 @@
       </c>
       <c r="K26" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1024</t>
+          <t>Pending commissioning - quality register 1024</t>
         </is>
       </c>
       <c r="L26" s="5" t="inlineStr">
@@ -2491,7 +2491,7 @@
       </c>
       <c r="K27" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1025</t>
+          <t>Pending commissioning - quality register 1025</t>
         </is>
       </c>
       <c r="L27" s="5" t="inlineStr">
@@ -2547,7 +2547,7 @@
       </c>
       <c r="K28" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1026</t>
+          <t>Pending commissioning - quality register 1026</t>
         </is>
       </c>
       <c r="L28" s="5" t="inlineStr">
@@ -2603,7 +2603,7 @@
       </c>
       <c r="K29" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1027</t>
+          <t>Pending commissioning - quality register 1027</t>
         </is>
       </c>
       <c r="L29" s="5" t="inlineStr">
@@ -2659,7 +2659,7 @@
       </c>
       <c r="K30" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1028</t>
+          <t>Pending commissioning - quality register 1028</t>
         </is>
       </c>
       <c r="L30" s="5" t="inlineStr">
@@ -2715,7 +2715,7 @@
       </c>
       <c r="K31" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1029</t>
+          <t>Pending commissioning - quality register 1029</t>
         </is>
       </c>
       <c r="L31" s="5" t="inlineStr">
@@ -2771,7 +2771,7 @@
       </c>
       <c r="K32" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1030</t>
+          <t>Pending commissioning - quality register 1030</t>
         </is>
       </c>
       <c r="L32" s="5" t="inlineStr">
@@ -2827,7 +2827,7 @@
       </c>
       <c r="K33" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1031</t>
+          <t>Pending commissioning - quality register 1031</t>
         </is>
       </c>
       <c r="L33" s="5" t="inlineStr">
@@ -2883,7 +2883,7 @@
       </c>
       <c r="K34" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1032</t>
+          <t>Pending commissioning - quality register 1032</t>
         </is>
       </c>
       <c r="L34" s="5" t="inlineStr">
@@ -2939,7 +2939,7 @@
       </c>
       <c r="K35" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1033</t>
+          <t>Pending commissioning - quality register 1033</t>
         </is>
       </c>
       <c r="L35" s="5" t="inlineStr">
@@ -2995,7 +2995,7 @@
       </c>
       <c r="K36" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1034</t>
+          <t>Pending commissioning - quality register 1034</t>
         </is>
       </c>
       <c r="L36" s="5" t="inlineStr">
@@ -3051,7 +3051,7 @@
       </c>
       <c r="K37" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1035</t>
+          <t>Pending commissioning - quality register 1035</t>
         </is>
       </c>
       <c r="L37" s="5" t="inlineStr">
@@ -3107,7 +3107,7 @@
       </c>
       <c r="K38" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1036</t>
+          <t>Pending commissioning - quality register 1036</t>
         </is>
       </c>
       <c r="L38" s="5" t="inlineStr">
@@ -3163,7 +3163,7 @@
       </c>
       <c r="K39" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1037</t>
+          <t>Pending commissioning - quality register 1037</t>
         </is>
       </c>
       <c r="L39" s="5" t="inlineStr">
@@ -3219,7 +3219,7 @@
       </c>
       <c r="K40" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1038</t>
+          <t>Pending commissioning - quality register 1038</t>
         </is>
       </c>
       <c r="L40" s="5" t="inlineStr">
@@ -3271,7 +3271,7 @@
       </c>
       <c r="K41" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1039</t>
+          <t>Pending commissioning - quality register 1039</t>
         </is>
       </c>
       <c r="L41" s="5" t="inlineStr">
@@ -3327,7 +3327,7 @@
       </c>
       <c r="K42" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1040</t>
+          <t>Pending commissioning - quality register 1040</t>
         </is>
       </c>
       <c r="L42" s="5" t="inlineStr">
@@ -3383,7 +3383,7 @@
       </c>
       <c r="K43" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1041</t>
+          <t>Pending commissioning - quality register 1041</t>
         </is>
       </c>
       <c r="L43" s="5" t="inlineStr">
@@ -3439,7 +3439,7 @@
       </c>
       <c r="K44" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1042</t>
+          <t>Pending commissioning - quality register 1042</t>
         </is>
       </c>
       <c r="L44" s="5" t="inlineStr">
@@ -3495,7 +3495,7 @@
       </c>
       <c r="K45" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1043</t>
+          <t>Pending commissioning - quality register 1043</t>
         </is>
       </c>
       <c r="L45" s="5" t="inlineStr">
@@ -3551,7 +3551,7 @@
       </c>
       <c r="K46" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1044</t>
+          <t>Pending commissioning - quality register 1044</t>
         </is>
       </c>
       <c r="L46" s="5" t="inlineStr">
@@ -3607,7 +3607,7 @@
       </c>
       <c r="K47" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1045</t>
+          <t>Pending commissioning - quality register 1045</t>
         </is>
       </c>
       <c r="L47" s="5" t="inlineStr">
@@ -3663,7 +3663,7 @@
       </c>
       <c r="K48" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1046</t>
+          <t>Pending commissioning - quality register 1046</t>
         </is>
       </c>
       <c r="L48" s="5" t="inlineStr">
@@ -3719,7 +3719,7 @@
       </c>
       <c r="K49" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1047</t>
+          <t>Pending commissioning - quality register 1047</t>
         </is>
       </c>
       <c r="L49" s="5" t="inlineStr">
@@ -3775,7 +3775,7 @@
       </c>
       <c r="K50" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1048</t>
+          <t>Pending commissioning - quality register 1048</t>
         </is>
       </c>
       <c r="L50" s="5" t="inlineStr">
@@ -3831,7 +3831,7 @@
       </c>
       <c r="K51" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1049</t>
+          <t>Pending commissioning - quality register 1049</t>
         </is>
       </c>
       <c r="L51" s="5" t="inlineStr">
@@ -3887,7 +3887,7 @@
       </c>
       <c r="K52" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1050</t>
+          <t>Pending commissioning - quality register 1050</t>
         </is>
       </c>
       <c r="L52" s="5" t="inlineStr">
@@ -3943,7 +3943,7 @@
       </c>
       <c r="K53" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1051</t>
+          <t>Pending commissioning - quality register 1051</t>
         </is>
       </c>
       <c r="L53" s="5" t="inlineStr">
@@ -3999,7 +3999,7 @@
       </c>
       <c r="K54" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1052</t>
+          <t>Pending commissioning - quality register 1052</t>
         </is>
       </c>
       <c r="L54" s="5" t="inlineStr">
@@ -4055,7 +4055,7 @@
       </c>
       <c r="K55" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1053</t>
+          <t>Pending commissioning - quality register 1053</t>
         </is>
       </c>
       <c r="L55" s="5" t="inlineStr">
@@ -4111,7 +4111,7 @@
       </c>
       <c r="K56" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1054</t>
+          <t>Pending commissioning - quality register 1054</t>
         </is>
       </c>
       <c r="L56" s="5" t="inlineStr">
@@ -4167,7 +4167,7 @@
       </c>
       <c r="K57" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1055</t>
+          <t>Pending commissioning - quality register 1055</t>
         </is>
       </c>
       <c r="L57" s="5" t="inlineStr">
@@ -4223,7 +4223,7 @@
       </c>
       <c r="K58" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1056</t>
+          <t>Pending commissioning - quality register 1056</t>
         </is>
       </c>
       <c r="L58" s="5" t="inlineStr">
@@ -4279,7 +4279,7 @@
       </c>
       <c r="K59" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1057</t>
+          <t>Pending commissioning - quality register 1057</t>
         </is>
       </c>
       <c r="L59" s="5" t="inlineStr">
@@ -4335,7 +4335,7 @@
       </c>
       <c r="K60" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1058</t>
+          <t>Pending commissioning - quality register 1058</t>
         </is>
       </c>
       <c r="L60" s="5" t="inlineStr">
@@ -4391,7 +4391,7 @@
       </c>
       <c r="K61" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1059</t>
+          <t>Pending commissioning - quality register 1059</t>
         </is>
       </c>
       <c r="L61" s="5" t="inlineStr">
@@ -4447,7 +4447,7 @@
       </c>
       <c r="K62" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1060</t>
+          <t>Pending commissioning - quality register 1060</t>
         </is>
       </c>
       <c r="L62" s="5" t="inlineStr">
@@ -4503,7 +4503,7 @@
       </c>
       <c r="K63" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1061</t>
+          <t>Pending commissioning - quality register 1061</t>
         </is>
       </c>
       <c r="L63" s="5" t="inlineStr">
@@ -4559,7 +4559,7 @@
       </c>
       <c r="K64" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1062</t>
+          <t>Pending commissioning - quality register 1062</t>
         </is>
       </c>
       <c r="L64" s="5" t="inlineStr">
@@ -4615,7 +4615,7 @@
       </c>
       <c r="K65" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1063</t>
+          <t>Pending commissioning - quality register 1063</t>
         </is>
       </c>
       <c r="L65" s="5" t="inlineStr">
@@ -4671,7 +4671,7 @@
       </c>
       <c r="K66" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1064</t>
+          <t>Pending commissioning - quality register 1064</t>
         </is>
       </c>
       <c r="L66" s="5" t="inlineStr">
@@ -4727,7 +4727,7 @@
       </c>
       <c r="K67" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1065</t>
+          <t>Pending commissioning - quality register 1065</t>
         </is>
       </c>
       <c r="L67" s="5" t="inlineStr">
@@ -4783,7 +4783,7 @@
       </c>
       <c r="K68" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1066</t>
+          <t>Pending commissioning - quality register 1066</t>
         </is>
       </c>
       <c r="L68" s="5" t="inlineStr">
@@ -4839,7 +4839,7 @@
       </c>
       <c r="K69" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1067</t>
+          <t>Pending commissioning - quality register 1067</t>
         </is>
       </c>
       <c r="L69" s="5" t="inlineStr">
@@ -4891,7 +4891,7 @@
       </c>
       <c r="K70" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1068</t>
+          <t>Pending commissioning - quality register 1068</t>
         </is>
       </c>
       <c r="L70" s="5" t="inlineStr">
@@ -4947,7 +4947,7 @@
       </c>
       <c r="K71" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1069</t>
+          <t>Pending commissioning - quality register 1069</t>
         </is>
       </c>
       <c r="L71" s="5" t="inlineStr">
@@ -5003,7 +5003,7 @@
       </c>
       <c r="K72" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1070</t>
+          <t>Pending commissioning - quality register 1070</t>
         </is>
       </c>
       <c r="L72" s="5" t="inlineStr">
@@ -5059,7 +5059,7 @@
       </c>
       <c r="K73" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1071</t>
+          <t>Pending commissioning - quality register 1071</t>
         </is>
       </c>
       <c r="L73" s="5" t="inlineStr">
@@ -5115,7 +5115,7 @@
       </c>
       <c r="K74" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1072</t>
+          <t>Pending commissioning - quality register 1072</t>
         </is>
       </c>
       <c r="L74" s="5" t="inlineStr">
@@ -5171,7 +5171,7 @@
       </c>
       <c r="K75" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1073</t>
+          <t>Pending commissioning - quality register 1073</t>
         </is>
       </c>
       <c r="L75" s="5" t="inlineStr">
@@ -5227,7 +5227,7 @@
       </c>
       <c r="K76" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1074</t>
+          <t>Pending commissioning - quality register 1074</t>
         </is>
       </c>
       <c r="L76" s="5" t="inlineStr">
@@ -5283,7 +5283,7 @@
       </c>
       <c r="K77" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1075</t>
+          <t>Pending commissioning - quality register 1075</t>
         </is>
       </c>
       <c r="L77" s="5" t="inlineStr">
@@ -5339,7 +5339,7 @@
       </c>
       <c r="K78" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1076</t>
+          <t>Pending commissioning - quality register 1076</t>
         </is>
       </c>
       <c r="L78" s="5" t="inlineStr">
@@ -5395,7 +5395,7 @@
       </c>
       <c r="K79" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1077</t>
+          <t>Pending commissioning - quality register 1077</t>
         </is>
       </c>
       <c r="L79" s="5" t="inlineStr">
@@ -5451,7 +5451,7 @@
       </c>
       <c r="K80" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1078</t>
+          <t>Pending commissioning - quality register 1078</t>
         </is>
       </c>
       <c r="L80" s="5" t="inlineStr">
@@ -5507,7 +5507,7 @@
       </c>
       <c r="K81" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1079</t>
+          <t>Pending commissioning - quality register 1079</t>
         </is>
       </c>
       <c r="L81" s="5" t="inlineStr">
@@ -5563,7 +5563,7 @@
       </c>
       <c r="K82" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1080</t>
+          <t>Pending commissioning - quality register 1080</t>
         </is>
       </c>
       <c r="L82" s="5" t="inlineStr">
@@ -5619,7 +5619,7 @@
       </c>
       <c r="K83" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1081</t>
+          <t>Pending commissioning - quality register 1081</t>
         </is>
       </c>
       <c r="L83" s="5" t="inlineStr">
@@ -5675,7 +5675,7 @@
       </c>
       <c r="K84" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1082</t>
+          <t>Pending commissioning - quality register 1082</t>
         </is>
       </c>
       <c r="L84" s="5" t="inlineStr">
@@ -5731,7 +5731,7 @@
       </c>
       <c r="K85" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1083</t>
+          <t>Pending commissioning - quality register 1083</t>
         </is>
       </c>
       <c r="L85" s="5" t="inlineStr">
@@ -5787,7 +5787,7 @@
       </c>
       <c r="K86" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1084</t>
+          <t>Pending commissioning - quality register 1084</t>
         </is>
       </c>
       <c r="L86" s="5" t="inlineStr">
@@ -5843,7 +5843,7 @@
       </c>
       <c r="K87" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1085</t>
+          <t>Pending commissioning - quality register 1085</t>
         </is>
       </c>
       <c r="L87" s="5" t="inlineStr">
@@ -5899,7 +5899,7 @@
       </c>
       <c r="K88" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1086</t>
+          <t>Pending commissioning - quality register 1086</t>
         </is>
       </c>
       <c r="L88" s="5" t="inlineStr">
@@ -5955,7 +5955,7 @@
       </c>
       <c r="K89" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1087</t>
+          <t>Pending commissioning - quality register 1087</t>
         </is>
       </c>
       <c r="L89" s="5" t="inlineStr">
@@ -6011,7 +6011,7 @@
       </c>
       <c r="K90" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1088</t>
+          <t>Pending commissioning - quality register 1088</t>
         </is>
       </c>
       <c r="L90" s="5" t="inlineStr">
@@ -6067,7 +6067,7 @@
       </c>
       <c r="K91" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1089</t>
+          <t>Pending commissioning - quality register 1089</t>
         </is>
       </c>
       <c r="L91" s="5" t="inlineStr">
@@ -6123,7 +6123,7 @@
       </c>
       <c r="K92" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1090</t>
+          <t>Pending commissioning - quality register 1090</t>
         </is>
       </c>
       <c r="L92" s="5" t="inlineStr">
@@ -6179,7 +6179,7 @@
       </c>
       <c r="K93" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1091</t>
+          <t>Pending commissioning - quality register 1091</t>
         </is>
       </c>
       <c r="L93" s="5" t="inlineStr">
@@ -6235,7 +6235,7 @@
       </c>
       <c r="K94" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1092</t>
+          <t>Pending commissioning - quality register 1092</t>
         </is>
       </c>
       <c r="L94" s="5" t="inlineStr">
@@ -6291,7 +6291,7 @@
       </c>
       <c r="K95" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1093</t>
+          <t>Pending commissioning - quality register 1093</t>
         </is>
       </c>
       <c r="L95" s="5" t="inlineStr">
@@ -6347,7 +6347,7 @@
       </c>
       <c r="K96" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1094</t>
+          <t>Pending commissioning - quality register 1094</t>
         </is>
       </c>
       <c r="L96" s="5" t="inlineStr">
@@ -6403,7 +6403,7 @@
       </c>
       <c r="K97" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1095</t>
+          <t>Pending commissioning - quality register 1095</t>
         </is>
       </c>
       <c r="L97" s="5" t="inlineStr">
@@ -6459,7 +6459,7 @@
       </c>
       <c r="K98" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1096</t>
+          <t>Pending commissioning - quality register 1096</t>
         </is>
       </c>
       <c r="L98" s="5" t="inlineStr">
@@ -6511,7 +6511,7 @@
       </c>
       <c r="K99" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1097</t>
+          <t>Pending commissioning - quality register 1097</t>
         </is>
       </c>
       <c r="L99" s="5" t="inlineStr">
@@ -6567,7 +6567,7 @@
       </c>
       <c r="K100" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1098</t>
+          <t>Pending commissioning - quality register 1098</t>
         </is>
       </c>
       <c r="L100" s="5" t="inlineStr">
@@ -6623,7 +6623,7 @@
       </c>
       <c r="K101" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1099</t>
+          <t>Pending commissioning - quality register 1099</t>
         </is>
       </c>
       <c r="L101" s="5" t="inlineStr">
@@ -6679,7 +6679,7 @@
       </c>
       <c r="K102" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1100</t>
+          <t>Pending commissioning - quality register 1100</t>
         </is>
       </c>
       <c r="L102" s="5" t="inlineStr">
@@ -6735,7 +6735,7 @@
       </c>
       <c r="K103" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1101</t>
+          <t>Pending commissioning - quality register 1101</t>
         </is>
       </c>
       <c r="L103" s="5" t="inlineStr">
@@ -6791,7 +6791,7 @@
       </c>
       <c r="K104" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1102</t>
+          <t>Pending commissioning - quality register 1102</t>
         </is>
       </c>
       <c r="L104" s="5" t="inlineStr">
@@ -6847,7 +6847,7 @@
       </c>
       <c r="K105" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1103</t>
+          <t>Pending commissioning - quality register 1103</t>
         </is>
       </c>
       <c r="L105" s="5" t="inlineStr">
@@ -6903,7 +6903,7 @@
       </c>
       <c r="K106" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1104</t>
+          <t>Pending commissioning - quality register 1104</t>
         </is>
       </c>
       <c r="L106" s="5" t="inlineStr">
@@ -6959,7 +6959,7 @@
       </c>
       <c r="K107" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1105</t>
+          <t>Pending commissioning - quality register 1105</t>
         </is>
       </c>
       <c r="L107" s="5" t="inlineStr">
@@ -7015,7 +7015,7 @@
       </c>
       <c r="K108" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1106</t>
+          <t>Pending commissioning - quality register 1106</t>
         </is>
       </c>
       <c r="L108" s="5" t="inlineStr">
@@ -7071,7 +7071,7 @@
       </c>
       <c r="K109" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1107</t>
+          <t>Pending commissioning - quality register 1107</t>
         </is>
       </c>
       <c r="L109" s="5" t="inlineStr">
@@ -7127,7 +7127,7 @@
       </c>
       <c r="K110" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1108</t>
+          <t>Pending commissioning - quality register 1108</t>
         </is>
       </c>
       <c r="L110" s="5" t="inlineStr">
@@ -7183,7 +7183,7 @@
       </c>
       <c r="K111" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1109</t>
+          <t>Pending commissioning - quality register 1109</t>
         </is>
       </c>
       <c r="L111" s="5" t="inlineStr">
@@ -7239,7 +7239,7 @@
       </c>
       <c r="K112" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1110</t>
+          <t>Pending commissioning - quality register 1110</t>
         </is>
       </c>
       <c r="L112" s="5" t="inlineStr">
@@ -7295,7 +7295,7 @@
       </c>
       <c r="K113" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1111</t>
+          <t>Pending commissioning - quality register 1111</t>
         </is>
       </c>
       <c r="L113" s="5" t="inlineStr">
@@ -7351,7 +7351,7 @@
       </c>
       <c r="K114" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1112</t>
+          <t>Pending commissioning - quality register 1112</t>
         </is>
       </c>
       <c r="L114" s="5" t="inlineStr">
@@ -7407,7 +7407,7 @@
       </c>
       <c r="K115" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1113</t>
+          <t>Pending commissioning - quality register 1113</t>
         </is>
       </c>
       <c r="L115" s="5" t="inlineStr">
@@ -7463,7 +7463,7 @@
       </c>
       <c r="K116" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1114</t>
+          <t>Pending commissioning - quality register 1114</t>
         </is>
       </c>
       <c r="L116" s="5" t="inlineStr">
@@ -7519,7 +7519,7 @@
       </c>
       <c r="K117" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1115</t>
+          <t>Pending commissioning - quality register 1115</t>
         </is>
       </c>
       <c r="L117" s="5" t="inlineStr">
@@ -7575,7 +7575,7 @@
       </c>
       <c r="K118" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1116</t>
+          <t>Pending commissioning - quality register 1116</t>
         </is>
       </c>
       <c r="L118" s="5" t="inlineStr">
@@ -7631,7 +7631,7 @@
       </c>
       <c r="K119" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1117</t>
+          <t>Pending commissioning - quality register 1117</t>
         </is>
       </c>
       <c r="L119" s="5" t="inlineStr">
@@ -7687,7 +7687,7 @@
       </c>
       <c r="K120" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1118</t>
+          <t>Pending commissioning - quality register 1118</t>
         </is>
       </c>
       <c r="L120" s="5" t="inlineStr">
@@ -7743,7 +7743,7 @@
       </c>
       <c r="K121" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1119</t>
+          <t>Pending commissioning - quality register 1119</t>
         </is>
       </c>
       <c r="L121" s="5" t="inlineStr">
@@ -7799,7 +7799,7 @@
       </c>
       <c r="K122" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1120</t>
+          <t>Pending commissioning - quality register 1120</t>
         </is>
       </c>
       <c r="L122" s="5" t="inlineStr">
@@ -7855,7 +7855,7 @@
       </c>
       <c r="K123" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1121</t>
+          <t>Pending commissioning - quality register 1121</t>
         </is>
       </c>
       <c r="L123" s="5" t="inlineStr">
@@ -7911,7 +7911,7 @@
       </c>
       <c r="K124" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1122</t>
+          <t>Pending commissioning - quality register 1122</t>
         </is>
       </c>
       <c r="L124" s="5" t="inlineStr">
@@ -7967,7 +7967,7 @@
       </c>
       <c r="K125" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1123</t>
+          <t>Pending commissioning - quality register 1123</t>
         </is>
       </c>
       <c r="L125" s="5" t="inlineStr">
@@ -8023,7 +8023,7 @@
       </c>
       <c r="K126" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1124</t>
+          <t>Pending commissioning - quality register 1124</t>
         </is>
       </c>
       <c r="L126" s="5" t="inlineStr">
@@ -8079,7 +8079,7 @@
       </c>
       <c r="K127" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1125</t>
+          <t>Pending commissioning - quality register 1125</t>
         </is>
       </c>
       <c r="L127" s="5" t="inlineStr">
@@ -8131,7 +8131,7 @@
       </c>
       <c r="K128" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1126</t>
+          <t>Pending commissioning - quality register 1126</t>
         </is>
       </c>
       <c r="L128" s="5" t="inlineStr">
@@ -8187,7 +8187,7 @@
       </c>
       <c r="K129" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1127</t>
+          <t>Pending commissioning - quality register 1127</t>
         </is>
       </c>
       <c r="L129" s="5" t="inlineStr">
@@ -8243,7 +8243,7 @@
       </c>
       <c r="K130" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1128</t>
+          <t>Pending commissioning - quality register 1128</t>
         </is>
       </c>
       <c r="L130" s="5" t="inlineStr">
@@ -8299,7 +8299,7 @@
       </c>
       <c r="K131" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1129</t>
+          <t>Pending commissioning - quality register 1129</t>
         </is>
       </c>
       <c r="L131" s="5" t="inlineStr">
@@ -8355,7 +8355,7 @@
       </c>
       <c r="K132" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1130</t>
+          <t>Pending commissioning - quality register 1130</t>
         </is>
       </c>
       <c r="L132" s="5" t="inlineStr">
@@ -8411,7 +8411,7 @@
       </c>
       <c r="K133" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1131</t>
+          <t>Pending commissioning - quality register 1131</t>
         </is>
       </c>
       <c r="L133" s="5" t="inlineStr">
@@ -8467,7 +8467,7 @@
       </c>
       <c r="K134" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1132</t>
+          <t>Pending commissioning - quality register 1132</t>
         </is>
       </c>
       <c r="L134" s="5" t="inlineStr">
@@ -8523,7 +8523,7 @@
       </c>
       <c r="K135" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1133</t>
+          <t>Pending commissioning - quality register 1133</t>
         </is>
       </c>
       <c r="L135" s="5" t="inlineStr">
@@ -8579,7 +8579,7 @@
       </c>
       <c r="K136" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1134</t>
+          <t>Pending commissioning - quality register 1134</t>
         </is>
       </c>
       <c r="L136" s="5" t="inlineStr">
@@ -8635,7 +8635,7 @@
       </c>
       <c r="K137" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1135</t>
+          <t>Pending commissioning - quality register 1135</t>
         </is>
       </c>
       <c r="L137" s="5" t="inlineStr">
@@ -8691,7 +8691,7 @@
       </c>
       <c r="K138" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1136</t>
+          <t>Pending commissioning - quality register 1136</t>
         </is>
       </c>
       <c r="L138" s="5" t="inlineStr">
@@ -8747,7 +8747,7 @@
       </c>
       <c r="K139" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1137</t>
+          <t>Pending commissioning - quality register 1137</t>
         </is>
       </c>
       <c r="L139" s="5" t="inlineStr">
@@ -8803,7 +8803,7 @@
       </c>
       <c r="K140" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1138</t>
+          <t>Pending commissioning - quality register 1138</t>
         </is>
       </c>
       <c r="L140" s="5" t="inlineStr">
@@ -8859,7 +8859,7 @@
       </c>
       <c r="K141" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1139</t>
+          <t>Pending commissioning - quality register 1139</t>
         </is>
       </c>
       <c r="L141" s="5" t="inlineStr">
@@ -8915,7 +8915,7 @@
       </c>
       <c r="K142" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1140</t>
+          <t>Pending commissioning - quality register 1140</t>
         </is>
       </c>
       <c r="L142" s="5" t="inlineStr">
@@ -8971,7 +8971,7 @@
       </c>
       <c r="K143" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1141</t>
+          <t>Pending commissioning - quality register 1141</t>
         </is>
       </c>
       <c r="L143" s="5" t="inlineStr">
@@ -9027,7 +9027,7 @@
       </c>
       <c r="K144" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1142</t>
+          <t>Pending commissioning - quality register 1142</t>
         </is>
       </c>
       <c r="L144" s="5" t="inlineStr">
@@ -9083,7 +9083,7 @@
       </c>
       <c r="K145" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1143</t>
+          <t>Pending commissioning - quality register 1143</t>
         </is>
       </c>
       <c r="L145" s="5" t="inlineStr">
@@ -9139,7 +9139,7 @@
       </c>
       <c r="K146" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1144</t>
+          <t>Pending commissioning - quality register 1144</t>
         </is>
       </c>
       <c r="L146" s="5" t="inlineStr">
@@ -9195,7 +9195,7 @@
       </c>
       <c r="K147" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1145</t>
+          <t>Pending commissioning - quality register 1145</t>
         </is>
       </c>
       <c r="L147" s="5" t="inlineStr">
@@ -9251,7 +9251,7 @@
       </c>
       <c r="K148" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1146</t>
+          <t>Pending commissioning - quality register 1146</t>
         </is>
       </c>
       <c r="L148" s="5" t="inlineStr">
@@ -9307,7 +9307,7 @@
       </c>
       <c r="K149" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1147</t>
+          <t>Pending commissioning - quality register 1147</t>
         </is>
       </c>
       <c r="L149" s="5" t="inlineStr">
@@ -9363,7 +9363,7 @@
       </c>
       <c r="K150" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1148</t>
+          <t>Pending commissioning - quality register 1148</t>
         </is>
       </c>
       <c r="L150" s="5" t="inlineStr">
@@ -9419,7 +9419,7 @@
       </c>
       <c r="K151" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1149</t>
+          <t>Pending commissioning - quality register 1149</t>
         </is>
       </c>
       <c r="L151" s="5" t="inlineStr">
@@ -9475,7 +9475,7 @@
       </c>
       <c r="K152" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1150</t>
+          <t>Pending commissioning - quality register 1150</t>
         </is>
       </c>
       <c r="L152" s="5" t="inlineStr">
@@ -9531,7 +9531,7 @@
       </c>
       <c r="K153" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1151</t>
+          <t>Pending commissioning - quality register 1151</t>
         </is>
       </c>
       <c r="L153" s="5" t="inlineStr">
@@ -9587,7 +9587,7 @@
       </c>
       <c r="K154" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1152</t>
+          <t>Pending commissioning - quality register 1152</t>
         </is>
       </c>
       <c r="L154" s="5" t="inlineStr">
@@ -9643,7 +9643,7 @@
       </c>
       <c r="K155" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1153</t>
+          <t>Pending commissioning - quality register 1153</t>
         </is>
       </c>
       <c r="L155" s="5" t="inlineStr">
@@ -9699,7 +9699,7 @@
       </c>
       <c r="K156" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1154</t>
+          <t>Pending commissioning - quality register 1154</t>
         </is>
       </c>
       <c r="L156" s="5" t="inlineStr">
@@ -9751,7 +9751,7 @@
       </c>
       <c r="K157" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1155</t>
+          <t>Pending commissioning - quality register 1155</t>
         </is>
       </c>
       <c r="L157" s="5" t="inlineStr">
@@ -9807,7 +9807,7 @@
       </c>
       <c r="K158" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1156</t>
+          <t>Pending commissioning - quality register 1156</t>
         </is>
       </c>
       <c r="L158" s="5" t="inlineStr">
@@ -9863,7 +9863,7 @@
       </c>
       <c r="K159" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1157</t>
+          <t>Pending commissioning - quality register 1157</t>
         </is>
       </c>
       <c r="L159" s="5" t="inlineStr">
@@ -9919,7 +9919,7 @@
       </c>
       <c r="K160" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1158</t>
+          <t>Pending commissioning - quality register 1158</t>
         </is>
       </c>
       <c r="L160" s="5" t="inlineStr">
@@ -9975,7 +9975,7 @@
       </c>
       <c r="K161" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1159</t>
+          <t>Pending commissioning - quality register 1159</t>
         </is>
       </c>
       <c r="L161" s="5" t="inlineStr">
@@ -10031,7 +10031,7 @@
       </c>
       <c r="K162" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1160</t>
+          <t>Pending commissioning - quality register 1160</t>
         </is>
       </c>
       <c r="L162" s="5" t="inlineStr">
@@ -10087,7 +10087,7 @@
       </c>
       <c r="K163" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1161</t>
+          <t>Pending commissioning - quality register 1161</t>
         </is>
       </c>
       <c r="L163" s="5" t="inlineStr">
@@ -10143,7 +10143,7 @@
       </c>
       <c r="K164" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1162</t>
+          <t>Pending commissioning - quality register 1162</t>
         </is>
       </c>
       <c r="L164" s="5" t="inlineStr">
@@ -10199,7 +10199,7 @@
       </c>
       <c r="K165" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1163</t>
+          <t>Pending commissioning - quality register 1163</t>
         </is>
       </c>
       <c r="L165" s="5" t="inlineStr">
@@ -10255,7 +10255,7 @@
       </c>
       <c r="K166" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1164</t>
+          <t>Pending commissioning - quality register 1164</t>
         </is>
       </c>
       <c r="L166" s="5" t="inlineStr">
@@ -10311,7 +10311,7 @@
       </c>
       <c r="K167" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1165</t>
+          <t>Pending commissioning - quality register 1165</t>
         </is>
       </c>
       <c r="L167" s="5" t="inlineStr">
@@ -10367,7 +10367,7 @@
       </c>
       <c r="K168" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1166</t>
+          <t>Pending commissioning - quality register 1166</t>
         </is>
       </c>
       <c r="L168" s="5" t="inlineStr">
@@ -10423,7 +10423,7 @@
       </c>
       <c r="K169" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1167</t>
+          <t>Pending commissioning - quality register 1167</t>
         </is>
       </c>
       <c r="L169" s="5" t="inlineStr">
@@ -10479,7 +10479,7 @@
       </c>
       <c r="K170" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1168</t>
+          <t>Pending commissioning - quality register 1168</t>
         </is>
       </c>
       <c r="L170" s="5" t="inlineStr">
@@ -10535,7 +10535,7 @@
       </c>
       <c r="K171" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1169</t>
+          <t>Pending commissioning - quality register 1169</t>
         </is>
       </c>
       <c r="L171" s="5" t="inlineStr">
@@ -10591,7 +10591,7 @@
       </c>
       <c r="K172" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1170</t>
+          <t>Pending commissioning - quality register 1170</t>
         </is>
       </c>
       <c r="L172" s="5" t="inlineStr">
@@ -10647,7 +10647,7 @@
       </c>
       <c r="K173" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1171</t>
+          <t>Pending commissioning - quality register 1171</t>
         </is>
       </c>
       <c r="L173" s="5" t="inlineStr">
@@ -10703,7 +10703,7 @@
       </c>
       <c r="K174" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1172</t>
+          <t>Pending commissioning - quality register 1172</t>
         </is>
       </c>
       <c r="L174" s="5" t="inlineStr">
@@ -10759,7 +10759,7 @@
       </c>
       <c r="K175" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1173</t>
+          <t>Pending commissioning - quality register 1173</t>
         </is>
       </c>
       <c r="L175" s="5" t="inlineStr">
@@ -10815,7 +10815,7 @@
       </c>
       <c r="K176" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1174</t>
+          <t>Pending commissioning - quality register 1174</t>
         </is>
       </c>
       <c r="L176" s="5" t="inlineStr">
@@ -10871,7 +10871,7 @@
       </c>
       <c r="K177" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1175</t>
+          <t>Pending commissioning - quality register 1175</t>
         </is>
       </c>
       <c r="L177" s="5" t="inlineStr">
@@ -10927,7 +10927,7 @@
       </c>
       <c r="K178" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1176</t>
+          <t>Pending commissioning - quality register 1176</t>
         </is>
       </c>
       <c r="L178" s="5" t="inlineStr">
@@ -10983,7 +10983,7 @@
       </c>
       <c r="K179" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1177</t>
+          <t>Pending commissioning - quality register 1177</t>
         </is>
       </c>
       <c r="L179" s="5" t="inlineStr">
@@ -11039,7 +11039,7 @@
       </c>
       <c r="K180" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1178</t>
+          <t>Pending commissioning - quality register 1178</t>
         </is>
       </c>
       <c r="L180" s="5" t="inlineStr">
@@ -11095,7 +11095,7 @@
       </c>
       <c r="K181" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1179</t>
+          <t>Pending commissioning - quality register 1179</t>
         </is>
       </c>
       <c r="L181" s="5" t="inlineStr">
@@ -11151,7 +11151,7 @@
       </c>
       <c r="K182" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1180</t>
+          <t>Pending commissioning - quality register 1180</t>
         </is>
       </c>
       <c r="L182" s="5" t="inlineStr">
@@ -11207,7 +11207,7 @@
       </c>
       <c r="K183" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1181</t>
+          <t>Pending commissioning - quality register 1181</t>
         </is>
       </c>
       <c r="L183" s="5" t="inlineStr">
@@ -11263,7 +11263,7 @@
       </c>
       <c r="K184" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1182</t>
+          <t>Pending commissioning - quality register 1182</t>
         </is>
       </c>
       <c r="L184" s="5" t="inlineStr">
@@ -11319,7 +11319,7 @@
       </c>
       <c r="K185" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1183</t>
+          <t>Pending commissioning - quality register 1183</t>
         </is>
       </c>
       <c r="L185" s="5" t="inlineStr">
@@ -11371,7 +11371,7 @@
       </c>
       <c r="K186" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1184</t>
+          <t>Pending commissioning - quality register 1184</t>
         </is>
       </c>
       <c r="L186" s="5" t="inlineStr">
@@ -11427,7 +11427,7 @@
       </c>
       <c r="K187" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1185</t>
+          <t>Pending commissioning - quality register 1185</t>
         </is>
       </c>
       <c r="L187" s="5" t="inlineStr">
@@ -11483,7 +11483,7 @@
       </c>
       <c r="K188" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1186</t>
+          <t>Pending commissioning - quality register 1186</t>
         </is>
       </c>
       <c r="L188" s="5" t="inlineStr">
@@ -11539,7 +11539,7 @@
       </c>
       <c r="K189" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1187</t>
+          <t>Pending commissioning - quality register 1187</t>
         </is>
       </c>
       <c r="L189" s="5" t="inlineStr">
@@ -11595,7 +11595,7 @@
       </c>
       <c r="K190" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1188</t>
+          <t>Pending commissioning - quality register 1188</t>
         </is>
       </c>
       <c r="L190" s="5" t="inlineStr">
@@ -11651,7 +11651,7 @@
       </c>
       <c r="K191" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1189</t>
+          <t>Pending commissioning - quality register 1189</t>
         </is>
       </c>
       <c r="L191" s="5" t="inlineStr">
@@ -11707,7 +11707,7 @@
       </c>
       <c r="K192" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1190</t>
+          <t>Pending commissioning - quality register 1190</t>
         </is>
       </c>
       <c r="L192" s="5" t="inlineStr">
@@ -11763,7 +11763,7 @@
       </c>
       <c r="K193" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1191</t>
+          <t>Pending commissioning - quality register 1191</t>
         </is>
       </c>
       <c r="L193" s="5" t="inlineStr">
@@ -11819,7 +11819,7 @@
       </c>
       <c r="K194" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1192</t>
+          <t>Pending commissioning - quality register 1192</t>
         </is>
       </c>
       <c r="L194" s="5" t="inlineStr">
@@ -11875,7 +11875,7 @@
       </c>
       <c r="K195" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1193</t>
+          <t>Pending commissioning - quality register 1193</t>
         </is>
       </c>
       <c r="L195" s="5" t="inlineStr">
@@ -11931,7 +11931,7 @@
       </c>
       <c r="K196" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1194</t>
+          <t>Pending commissioning - quality register 1194</t>
         </is>
       </c>
       <c r="L196" s="5" t="inlineStr">
@@ -11987,7 +11987,7 @@
       </c>
       <c r="K197" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1195</t>
+          <t>Pending commissioning - quality register 1195</t>
         </is>
       </c>
       <c r="L197" s="5" t="inlineStr">
@@ -12043,7 +12043,7 @@
       </c>
       <c r="K198" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1196</t>
+          <t>Pending commissioning - quality register 1196</t>
         </is>
       </c>
       <c r="L198" s="5" t="inlineStr">
@@ -12099,7 +12099,7 @@
       </c>
       <c r="K199" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1197</t>
+          <t>Pending commissioning - quality register 1197</t>
         </is>
       </c>
       <c r="L199" s="5" t="inlineStr">
@@ -12155,7 +12155,7 @@
       </c>
       <c r="K200" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1198</t>
+          <t>Pending commissioning - quality register 1198</t>
         </is>
       </c>
       <c r="L200" s="5" t="inlineStr">
@@ -12211,7 +12211,7 @@
       </c>
       <c r="K201" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1199</t>
+          <t>Pending commissioning - quality register 1199</t>
         </is>
       </c>
       <c r="L201" s="5" t="inlineStr">
@@ -12267,7 +12267,7 @@
       </c>
       <c r="K202" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1200</t>
+          <t>Pending commissioning - quality register 1200</t>
         </is>
       </c>
       <c r="L202" s="5" t="inlineStr">
@@ -12323,7 +12323,7 @@
       </c>
       <c r="K203" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1201</t>
+          <t>Pending commissioning - quality register 1201</t>
         </is>
       </c>
       <c r="L203" s="5" t="inlineStr">
@@ -12379,7 +12379,7 @@
       </c>
       <c r="K204" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1202</t>
+          <t>Pending commissioning - quality register 1202</t>
         </is>
       </c>
       <c r="L204" s="5" t="inlineStr">
@@ -12435,7 +12435,7 @@
       </c>
       <c r="K205" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1203</t>
+          <t>Pending commissioning - quality register 1203</t>
         </is>
       </c>
       <c r="L205" s="5" t="inlineStr">
@@ -12491,7 +12491,7 @@
       </c>
       <c r="K206" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1204</t>
+          <t>Pending commissioning - quality register 1204</t>
         </is>
       </c>
       <c r="L206" s="5" t="inlineStr">
@@ -12547,7 +12547,7 @@
       </c>
       <c r="K207" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1205</t>
+          <t>Pending commissioning - quality register 1205</t>
         </is>
       </c>
       <c r="L207" s="5" t="inlineStr">
@@ -12603,7 +12603,7 @@
       </c>
       <c r="K208" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1206</t>
+          <t>Pending commissioning - quality register 1206</t>
         </is>
       </c>
       <c r="L208" s="5" t="inlineStr">
@@ -12659,7 +12659,7 @@
       </c>
       <c r="K209" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1207</t>
+          <t>Pending commissioning - quality register 1207</t>
         </is>
       </c>
       <c r="L209" s="5" t="inlineStr">
@@ -12715,7 +12715,7 @@
       </c>
       <c r="K210" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1208</t>
+          <t>Pending commissioning - quality register 1208</t>
         </is>
       </c>
       <c r="L210" s="5" t="inlineStr">
@@ -12771,7 +12771,7 @@
       </c>
       <c r="K211" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1209</t>
+          <t>Pending commissioning - quality register 1209</t>
         </is>
       </c>
       <c r="L211" s="5" t="inlineStr">
@@ -12827,7 +12827,7 @@
       </c>
       <c r="K212" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1210</t>
+          <t>Pending commissioning - quality register 1210</t>
         </is>
       </c>
       <c r="L212" s="5" t="inlineStr">
@@ -12883,7 +12883,7 @@
       </c>
       <c r="K213" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1211</t>
+          <t>Pending commissioning - quality register 1211</t>
         </is>
       </c>
       <c r="L213" s="5" t="inlineStr">
@@ -12939,7 +12939,7 @@
       </c>
       <c r="K214" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1212</t>
+          <t>Pending commissioning - quality register 1212</t>
         </is>
       </c>
       <c r="L214" s="5" t="inlineStr">
@@ -12991,7 +12991,7 @@
       </c>
       <c r="K215" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1213</t>
+          <t>Pending commissioning - quality register 1213</t>
         </is>
       </c>
       <c r="L215" s="5" t="inlineStr">
@@ -13047,7 +13047,7 @@
       </c>
       <c r="K216" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1214</t>
+          <t>Pending commissioning - quality register 1214</t>
         </is>
       </c>
       <c r="L216" s="5" t="inlineStr">
@@ -13103,7 +13103,7 @@
       </c>
       <c r="K217" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1215</t>
+          <t>Pending commissioning - quality register 1215</t>
         </is>
       </c>
       <c r="L217" s="5" t="inlineStr">
@@ -13159,7 +13159,7 @@
       </c>
       <c r="K218" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1216</t>
+          <t>Pending commissioning - quality register 1216</t>
         </is>
       </c>
       <c r="L218" s="5" t="inlineStr">
@@ -13215,7 +13215,7 @@
       </c>
       <c r="K219" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1217</t>
+          <t>Pending commissioning - quality register 1217</t>
         </is>
       </c>
       <c r="L219" s="5" t="inlineStr">
@@ -13271,7 +13271,7 @@
       </c>
       <c r="K220" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1218</t>
+          <t>Pending commissioning - quality register 1218</t>
         </is>
       </c>
       <c r="L220" s="5" t="inlineStr">
@@ -13327,7 +13327,7 @@
       </c>
       <c r="K221" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1219</t>
+          <t>Pending commissioning - quality register 1219</t>
         </is>
       </c>
       <c r="L221" s="5" t="inlineStr">
@@ -13383,7 +13383,7 @@
       </c>
       <c r="K222" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1220</t>
+          <t>Pending commissioning - quality register 1220</t>
         </is>
       </c>
       <c r="L222" s="5" t="inlineStr">
@@ -13439,7 +13439,7 @@
       </c>
       <c r="K223" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1221</t>
+          <t>Pending commissioning - quality register 1221</t>
         </is>
       </c>
       <c r="L223" s="5" t="inlineStr">
@@ -13495,7 +13495,7 @@
       </c>
       <c r="K224" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1222</t>
+          <t>Pending commissioning - quality register 1222</t>
         </is>
       </c>
       <c r="L224" s="5" t="inlineStr">
@@ -13551,7 +13551,7 @@
       </c>
       <c r="K225" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1223</t>
+          <t>Pending commissioning - quality register 1223</t>
         </is>
       </c>
       <c r="L225" s="5" t="inlineStr">
@@ -13607,7 +13607,7 @@
       </c>
       <c r="K226" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1224</t>
+          <t>Pending commissioning - quality register 1224</t>
         </is>
       </c>
       <c r="L226" s="5" t="inlineStr">
@@ -13663,7 +13663,7 @@
       </c>
       <c r="K227" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1225</t>
+          <t>Pending commissioning - quality register 1225</t>
         </is>
       </c>
       <c r="L227" s="5" t="inlineStr">
@@ -13719,7 +13719,7 @@
       </c>
       <c r="K228" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1226</t>
+          <t>Pending commissioning - quality register 1226</t>
         </is>
       </c>
       <c r="L228" s="5" t="inlineStr">
@@ -13775,7 +13775,7 @@
       </c>
       <c r="K229" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1227</t>
+          <t>Pending commissioning - quality register 1227</t>
         </is>
       </c>
       <c r="L229" s="5" t="inlineStr">
@@ -13831,7 +13831,7 @@
       </c>
       <c r="K230" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1228</t>
+          <t>Pending commissioning - quality register 1228</t>
         </is>
       </c>
       <c r="L230" s="5" t="inlineStr">
@@ -13887,7 +13887,7 @@
       </c>
       <c r="K231" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1229</t>
+          <t>Pending commissioning - quality register 1229</t>
         </is>
       </c>
       <c r="L231" s="5" t="inlineStr">
@@ -13943,7 +13943,7 @@
       </c>
       <c r="K232" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1230</t>
+          <t>Pending commissioning - quality register 1230</t>
         </is>
       </c>
       <c r="L232" s="5" t="inlineStr">
@@ -13999,7 +13999,7 @@
       </c>
       <c r="K233" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1231</t>
+          <t>Pending commissioning - quality register 1231</t>
         </is>
       </c>
       <c r="L233" s="5" t="inlineStr">
@@ -14055,7 +14055,7 @@
       </c>
       <c r="K234" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1232</t>
+          <t>Pending commissioning - quality register 1232</t>
         </is>
       </c>
       <c r="L234" s="5" t="inlineStr">
@@ -14111,7 +14111,7 @@
       </c>
       <c r="K235" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1233</t>
+          <t>Pending commissioning - quality register 1233</t>
         </is>
       </c>
       <c r="L235" s="5" t="inlineStr">
@@ -14167,7 +14167,7 @@
       </c>
       <c r="K236" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1234</t>
+          <t>Pending commissioning - quality register 1234</t>
         </is>
       </c>
       <c r="L236" s="5" t="inlineStr">
@@ -14223,7 +14223,7 @@
       </c>
       <c r="K237" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1235</t>
+          <t>Pending commissioning - quality register 1235</t>
         </is>
       </c>
       <c r="L237" s="5" t="inlineStr">
@@ -14279,7 +14279,7 @@
       </c>
       <c r="K238" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1236</t>
+          <t>Pending commissioning - quality register 1236</t>
         </is>
       </c>
       <c r="L238" s="5" t="inlineStr">
@@ -14335,7 +14335,7 @@
       </c>
       <c r="K239" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1237</t>
+          <t>Pending commissioning - quality register 1237</t>
         </is>
       </c>
       <c r="L239" s="5" t="inlineStr">
@@ -14391,7 +14391,7 @@
       </c>
       <c r="K240" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1238</t>
+          <t>Pending commissioning - quality register 1238</t>
         </is>
       </c>
       <c r="L240" s="5" t="inlineStr">
@@ -14447,7 +14447,7 @@
       </c>
       <c r="K241" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1239</t>
+          <t>Pending commissioning - quality register 1239</t>
         </is>
       </c>
       <c r="L241" s="5" t="inlineStr">
@@ -14503,7 +14503,7 @@
       </c>
       <c r="K242" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1240</t>
+          <t>Pending commissioning - quality register 1240</t>
         </is>
       </c>
       <c r="L242" s="5" t="inlineStr">
@@ -14559,7 +14559,7 @@
       </c>
       <c r="K243" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1241</t>
+          <t>Pending commissioning - quality register 1241</t>
         </is>
       </c>
       <c r="L243" s="5" t="inlineStr">
@@ -14611,7 +14611,7 @@
       </c>
       <c r="K244" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1242</t>
+          <t>Pending commissioning - quality register 1242</t>
         </is>
       </c>
       <c r="L244" s="5" t="inlineStr">
@@ -14667,7 +14667,7 @@
       </c>
       <c r="K245" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1243</t>
+          <t>Pending commissioning - quality register 1243</t>
         </is>
       </c>
       <c r="L245" s="5" t="inlineStr">
@@ -14723,7 +14723,7 @@
       </c>
       <c r="K246" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1244</t>
+          <t>Pending commissioning - quality register 1244</t>
         </is>
       </c>
       <c r="L246" s="5" t="inlineStr">
@@ -14779,7 +14779,7 @@
       </c>
       <c r="K247" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1245</t>
+          <t>Pending commissioning - quality register 1245</t>
         </is>
       </c>
       <c r="L247" s="5" t="inlineStr">
@@ -14835,7 +14835,7 @@
       </c>
       <c r="K248" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1246</t>
+          <t>Pending commissioning - quality register 1246</t>
         </is>
       </c>
       <c r="L248" s="5" t="inlineStr">
@@ -14891,7 +14891,7 @@
       </c>
       <c r="K249" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1247</t>
+          <t>Pending commissioning - quality register 1247</t>
         </is>
       </c>
       <c r="L249" s="5" t="inlineStr">
@@ -14947,7 +14947,7 @@
       </c>
       <c r="K250" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1248</t>
+          <t>Pending commissioning - quality register 1248</t>
         </is>
       </c>
       <c r="L250" s="5" t="inlineStr">
@@ -15003,7 +15003,7 @@
       </c>
       <c r="K251" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1249</t>
+          <t>Pending commissioning - quality register 1249</t>
         </is>
       </c>
       <c r="L251" s="5" t="inlineStr">
@@ -15059,7 +15059,7 @@
       </c>
       <c r="K252" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1250</t>
+          <t>Pending commissioning - quality register 1250</t>
         </is>
       </c>
       <c r="L252" s="5" t="inlineStr">
@@ -15115,7 +15115,7 @@
       </c>
       <c r="K253" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1251</t>
+          <t>Pending commissioning - quality register 1251</t>
         </is>
       </c>
       <c r="L253" s="5" t="inlineStr">
@@ -15171,7 +15171,7 @@
       </c>
       <c r="K254" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1252</t>
+          <t>Pending commissioning - quality register 1252</t>
         </is>
       </c>
       <c r="L254" s="5" t="inlineStr">
@@ -15227,7 +15227,7 @@
       </c>
       <c r="K255" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1253</t>
+          <t>Pending commissioning - quality register 1253</t>
         </is>
       </c>
       <c r="L255" s="5" t="inlineStr">
@@ -15283,7 +15283,7 @@
       </c>
       <c r="K256" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1254</t>
+          <t>Pending commissioning - quality register 1254</t>
         </is>
       </c>
       <c r="L256" s="5" t="inlineStr">
@@ -15339,7 +15339,7 @@
       </c>
       <c r="K257" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1255</t>
+          <t>Pending commissioning - quality register 1255</t>
         </is>
       </c>
       <c r="L257" s="5" t="inlineStr">
@@ -15395,7 +15395,7 @@
       </c>
       <c r="K258" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1256</t>
+          <t>Pending commissioning - quality register 1256</t>
         </is>
       </c>
       <c r="L258" s="5" t="inlineStr">
@@ -15451,7 +15451,7 @@
       </c>
       <c r="K259" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1257</t>
+          <t>Pending commissioning - quality register 1257</t>
         </is>
       </c>
       <c r="L259" s="5" t="inlineStr">
@@ -15507,7 +15507,7 @@
       </c>
       <c r="K260" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1258</t>
+          <t>Pending commissioning - quality register 1258</t>
         </is>
       </c>
       <c r="L260" s="5" t="inlineStr">
@@ -15563,7 +15563,7 @@
       </c>
       <c r="K261" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1259</t>
+          <t>Pending commissioning - quality register 1259</t>
         </is>
       </c>
       <c r="L261" s="5" t="inlineStr">
@@ -15619,7 +15619,7 @@
       </c>
       <c r="K262" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1260</t>
+          <t>Pending commissioning - quality register 1260</t>
         </is>
       </c>
       <c r="L262" s="5" t="inlineStr">
@@ -15675,7 +15675,7 @@
       </c>
       <c r="K263" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1261</t>
+          <t>Pending commissioning - quality register 1261</t>
         </is>
       </c>
       <c r="L263" s="5" t="inlineStr">
@@ -15731,7 +15731,7 @@
       </c>
       <c r="K264" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1262</t>
+          <t>Pending commissioning - quality register 1262</t>
         </is>
       </c>
       <c r="L264" s="5" t="inlineStr">
@@ -15787,7 +15787,7 @@
       </c>
       <c r="K265" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1263</t>
+          <t>Pending commissioning - quality register 1263</t>
         </is>
       </c>
       <c r="L265" s="5" t="inlineStr">
@@ -15843,7 +15843,7 @@
       </c>
       <c r="K266" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1264</t>
+          <t>Pending commissioning - quality register 1264</t>
         </is>
       </c>
       <c r="L266" s="5" t="inlineStr">
@@ -15899,7 +15899,7 @@
       </c>
       <c r="K267" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1265</t>
+          <t>Pending commissioning - quality register 1265</t>
         </is>
       </c>
       <c r="L267" s="5" t="inlineStr">
@@ -15955,7 +15955,7 @@
       </c>
       <c r="K268" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1266</t>
+          <t>Pending commissioning - quality register 1266</t>
         </is>
       </c>
       <c r="L268" s="5" t="inlineStr">
@@ -16011,7 +16011,7 @@
       </c>
       <c r="K269" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1267</t>
+          <t>Pending commissioning - quality register 1267</t>
         </is>
       </c>
       <c r="L269" s="5" t="inlineStr">
@@ -16067,7 +16067,7 @@
       </c>
       <c r="K270" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1268</t>
+          <t>Pending commissioning - quality register 1268</t>
         </is>
       </c>
       <c r="L270" s="5" t="inlineStr">
@@ -16123,7 +16123,7 @@
       </c>
       <c r="K271" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1269</t>
+          <t>Pending commissioning - quality register 1269</t>
         </is>
       </c>
       <c r="L271" s="5" t="inlineStr">
@@ -16179,7 +16179,7 @@
       </c>
       <c r="K272" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1270</t>
+          <t>Pending commissioning - quality register 1270</t>
         </is>
       </c>
       <c r="L272" s="5" t="inlineStr">
@@ -16231,7 +16231,7 @@
       </c>
       <c r="K273" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1271</t>
+          <t>Pending commissioning - quality register 1271</t>
         </is>
       </c>
       <c r="L273" s="5" t="inlineStr">
@@ -16287,7 +16287,7 @@
       </c>
       <c r="K274" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1272</t>
+          <t>Pending commissioning - quality register 1272</t>
         </is>
       </c>
       <c r="L274" s="5" t="inlineStr">
@@ -16343,7 +16343,7 @@
       </c>
       <c r="K275" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1273</t>
+          <t>Pending commissioning - quality register 1273</t>
         </is>
       </c>
       <c r="L275" s="5" t="inlineStr">
@@ -16399,7 +16399,7 @@
       </c>
       <c r="K276" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1274</t>
+          <t>Pending commissioning - quality register 1274</t>
         </is>
       </c>
       <c r="L276" s="5" t="inlineStr">
@@ -16455,7 +16455,7 @@
       </c>
       <c r="K277" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1275</t>
+          <t>Pending commissioning - quality register 1275</t>
         </is>
       </c>
       <c r="L277" s="5" t="inlineStr">
@@ -16511,7 +16511,7 @@
       </c>
       <c r="K278" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1276</t>
+          <t>Pending commissioning - quality register 1276</t>
         </is>
       </c>
       <c r="L278" s="5" t="inlineStr">
@@ -16567,7 +16567,7 @@
       </c>
       <c r="K279" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1277</t>
+          <t>Pending commissioning - quality register 1277</t>
         </is>
       </c>
       <c r="L279" s="5" t="inlineStr">
@@ -16623,7 +16623,7 @@
       </c>
       <c r="K280" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1278</t>
+          <t>Pending commissioning - quality register 1278</t>
         </is>
       </c>
       <c r="L280" s="5" t="inlineStr">
@@ -16679,7 +16679,7 @@
       </c>
       <c r="K281" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1279</t>
+          <t>Pending commissioning - quality register 1279</t>
         </is>
       </c>
       <c r="L281" s="5" t="inlineStr">
@@ -16735,7 +16735,7 @@
       </c>
       <c r="K282" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1280</t>
+          <t>Pending commissioning - quality register 1280</t>
         </is>
       </c>
       <c r="L282" s="5" t="inlineStr">
@@ -16791,7 +16791,7 @@
       </c>
       <c r="K283" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1281</t>
+          <t>Pending commissioning - quality register 1281</t>
         </is>
       </c>
       <c r="L283" s="5" t="inlineStr">
@@ -16847,7 +16847,7 @@
       </c>
       <c r="K284" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1282</t>
+          <t>Pending commissioning - quality register 1282</t>
         </is>
       </c>
       <c r="L284" s="5" t="inlineStr">
@@ -16903,7 +16903,7 @@
       </c>
       <c r="K285" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1283</t>
+          <t>Pending commissioning - quality register 1283</t>
         </is>
       </c>
       <c r="L285" s="5" t="inlineStr">
@@ -16959,7 +16959,7 @@
       </c>
       <c r="K286" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1284</t>
+          <t>Pending commissioning - quality register 1284</t>
         </is>
       </c>
       <c r="L286" s="5" t="inlineStr">
@@ -17015,7 +17015,7 @@
       </c>
       <c r="K287" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1285</t>
+          <t>Pending commissioning - quality register 1285</t>
         </is>
       </c>
       <c r="L287" s="5" t="inlineStr">
@@ -17071,7 +17071,7 @@
       </c>
       <c r="K288" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1286</t>
+          <t>Pending commissioning - quality register 1286</t>
         </is>
       </c>
       <c r="L288" s="5" t="inlineStr">
@@ -17127,7 +17127,7 @@
       </c>
       <c r="K289" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1287</t>
+          <t>Pending commissioning - quality register 1287</t>
         </is>
       </c>
       <c r="L289" s="5" t="inlineStr">
@@ -17183,7 +17183,7 @@
       </c>
       <c r="K290" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1288</t>
+          <t>Pending commissioning - quality register 1288</t>
         </is>
       </c>
       <c r="L290" s="5" t="inlineStr">
@@ -17239,7 +17239,7 @@
       </c>
       <c r="K291" s="6" t="inlineStr">
         <is>
-          <t>Pending - register map of the source device not yet available - quality register 1289</t>
+          <t>Pending commissioning - quality register 1289</t>
         </is>
       </c>
       <c r="L291" s="5" t="inlineStr">
@@ -17355,7 +17355,7 @@
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>Two energy meters (generator feeder, grid feeder), a PID device, a relay/RTU. No PV-side energy meter and no pyranometer / module temperature sensor on site.</t>
+          <t>Two energy meters (generator feeder, grid feeder), a PID device, a relay/RTU.</t>
         </is>
       </c>
     </row>
@@ -17415,7 +17415,7 @@
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>InteliNeo Modbus register table (2026-10-14), SAU device/signal export, InteliNeo history exports, integrator site-visit report (28.09.2026). Still needed: the SAU-100 Modbus TCP point table for the inverter signals</t>
+          <t>InteliNeo Modbus register table (2026-10-14), SAU device/signal export, InteliNeo history exports, integrator site-visit report (28.09.2026).</t>
         </is>
       </c>
     </row>
@@ -17439,7 +17439,7 @@
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>Rev.1.2 - 2026-10-14: PLC addresses are the plant-PC Modbus server addresses (fixed). Status column: Ready / Pending per tag.</t>
+          <t>Rev.1.2 - 2026-10-14: PLC addresses are the plant-PC Modbus server addresses (fixed). Status column: Ready / Pending commissioning per tag.</t>
         </is>
       </c>
     </row>
@@ -17470,7 +17470,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>Status column: Ready = the source signal is wired on site; Pending = the address is fixed but the value stays at quality 0 until the source device is mapped (inverters: SAU point table) or exists (PV-side meter, pyranometer, module temperature).</t>
+          <t>Status column: Ready = the source signal is already wired; Pending commissioning = the address is fixed, the value stays at quality 0 until commissioning of that signal is complete.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Turkey workbooks: NOTES sheet reduced to how to read the file and how to connect
</commit_message>
<xml_diff>
--- a/docs/turkey/Solar_Inverter_Tag_List_Rev.1.2.xlsx
+++ b/docs/turkey/Solar_Inverter_Tag_List_Rev.1.2.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="20">
+  <fonts count="21">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -144,6 +144,9 @@
     </font>
     <font>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="35">
@@ -512,7 +515,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -531,6 +534,7 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -17454,106 +17458,73 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A15"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="150" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="9" t="inlineStr">
+      <c r="A1" s="10" t="inlineStr">
         <is>
           <t>How to read this file</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="8" t="inlineStr">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>PLC_Address = the holding-register address on the plant-PC Modbus server (0-based, FC03). It is fixed and does not change during commissioning.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Float tags: float32, 2 registers, high word first (ABCD), engineering units, scale 1. Boolean tags: one register, 0 / 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Every tag has a quality register (see the register map): 1 = good, 2 = stale, 0 = not available.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
         <is>
           <t>Status column: Ready = the source signal is already wired; Pending commissioning = the address is fixed, the value stays at quality 0 until commissioning of that signal is complete.</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="8" t="inlineStr">
-        <is>
-          <t>PLC_Address = the holding-register address on the plant-PC Modbus server (0-based, FC03). It is fixed and does not change when the site-side device registers are mapped.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="8" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="9" t="inlineStr">
-        <is>
-          <t>Where the missing addresses come from</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="8" t="inlineStr">
-        <is>
-          <t>1. Inverter signals: the Sineng SAU-100 web UI exports the Modbus point table for the connected inverters (Setting → communication / point table). Alternatively the Sineng inverter Modbus protocol document for the installed model. Unit ID per inverter = the inverter's address on the SAU.</t>
-        </is>
-      </c>
-    </row>
+    <row r="6"/>
     <row r="7">
-      <c r="A7" s="8" t="inlineStr">
-        <is>
-          <t>2. Plant-level electrical signals (currents, voltages, P, Q, energy): from the electric meter connected to the SAU, or from the InteliNeo 5500 PV/bus measurements — whichever the site confirms as the official metering point.</t>
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>Architecture</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="inlineStr">
-        <is>
-          <t>3. Panel temperature / pyranometer: environmental sensors — confirm whether they are wired to the SAU (weather station input) or to another device.</t>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>One data collector on the plant PC reads the site devices (ComAp InteliNeo 5500 master controller, Sineng SAU-100 gateway) once per hour, read-only, and serves this list on its own Modbus TCP server. The monitoring platform connects to the plant PC only, never to the field devices.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="inlineStr">
-        <is>
-          <t>4. Breaker states (LV panel thermal-magnetic switch): PVCB status as seen by the InteliNeo (binary input) — register from the InteliConfig Modbus register export.</t>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Please poll the plant-PC server every 30-60 minutes in block reads (e.g. 100-699 and 1000-1304 in a few requests). The header registers 0-2 give the time of the last site read.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="inlineStr">
-        <is>
-          <t>5. ComAp values (PV prod, PV req, bus values, comm status): InteliConfig → Modules → Modbus Registers export of the InteliNeo configuration.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="8" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="9" t="inlineStr">
-        <is>
-          <t>IMPORTANT for the monitoring integration</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="8" t="inlineStr">
-        <is>
-          <t>The SAU Modbus TCP server is single-threaded and is already overloaded by the InteliNeo polling (two sessions, 0 ms pause). Comm-fail events in the InteliNeo cause PV anti-islanding trips and bus under-voltage. Adding another Modbus client directly on the SAU or the InteliNeo will make this worse.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="8" t="inlineStr">
-        <is>
-          <t>Recommended architecture: ONE local data collector on site reads the SAU and the InteliNeo gently (or reads the SCADA historian) and serves all consumers (DT Turkey monitoring, local dashboards) from its own database/OPC-UA/REST. No second poller on the field devices.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="8" t="inlineStr">
-        <is>
-          <t>Please poll the plant-PC server every 30-60 minutes in block reads (e.g. 100-699 and 1000-1304 in a few requests). The values refresh once per hour; the header registers 0-2 give the time of the last site read.</t>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Connection to the plant PC: through the CCI corporate network or a VPN account; the plant's public IP is not opened. Final IP address to follow once the method is agreed.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Turkey workbooks: contacts row
</commit_message>
<xml_diff>
--- a/docs/turkey/Solar_Inverter_Tag_List_Rev.1.2.xlsx
+++ b/docs/turkey/Solar_Inverter_Tag_List_Rev.1.2.xlsx
@@ -17419,7 +17419,7 @@
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>InteliNeo Modbus register table (2026-10-14), SAU device/signal export, InteliNeo history exports, integrator site-visit report (28.09.2026).</t>
+          <t>InteliNeo Modbus register table (2026-10-14), SAU device/signal export, InteliNeo history exports.</t>
         </is>
       </c>
     </row>
@@ -17431,7 +17431,7 @@
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>Eng. Yousif (site); Sabir (data / monitoring integration); Stromatik Automation, Eng. Salwan (ComAp integrator); Sineng support (via site)</t>
+          <t>Eng. Yousif (site); Sabir (data / monitoring integration)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Turkey workbooks: INFO wording
</commit_message>
<xml_diff>
--- a/docs/turkey/Solar_Inverter_Tag_List_Rev.1.2.xlsx
+++ b/docs/turkey/Solar_Inverter_Tag_List_Rev.1.2.xlsx
@@ -17371,7 +17371,7 @@
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>SAU local web UI (Device Monitor); ComAp InteliNeo 5500 master controller (IP 192.168.0.112) reads PV as 'PV Logger group 1/2' via Modbus TCP, unit address 245; plant SCADA PC; no cloud platform confirmed</t>
+          <t>SAU-100 local web interface (dashboard, device monitor, logs); ComAp InteliConfig on the plant computer for the controllers. The InteliNeo 5500 master controller (192.168.0.112) reads the PV totals from the SAU over Modbus TCP (unit address 245). No cloud platform connected.</t>
         </is>
       </c>
     </row>
@@ -17395,7 +17395,7 @@
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>Modbus TCP (SAU, InteliNeo); Modbus RTU (inverters ↔ SAU, RS485); ComAp AirGate/WebSupervisor possible for InteliNeo (not enabled yet)</t>
+          <t>Modbus TCP (SAU-100, InteliNeo); Modbus RTU over RS485 (inverters to SAU); the SAU also supports IEC 60870-5-104</t>
         </is>
       </c>
     </row>
@@ -17431,7 +17431,7 @@
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>Eng. Yousif (site); Sabir (data / monitoring integration)</t>
+          <t>Sabir Tishko (data / monitoring integration)</t>
         </is>
       </c>
     </row>
@@ -17499,7 +17499,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7">
       <c r="A7" s="10" t="inlineStr">
         <is>

</xml_diff>